<commit_message>
Clean across survey analysis files
</commit_message>
<xml_diff>
--- a/Across survey analysis/LPG and firewood statistics/TM - LPG analysis 4Apr25.xlsx
+++ b/Across survey analysis/LPG and firewood statistics/TM - LPG analysis 4Apr25.xlsx
@@ -9,17 +9,19 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15530" windowHeight="6930" firstSheet="4" activeTab="6"/>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6930" firstSheet="4" activeTab="6"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15525" windowHeight="6930" firstSheet="4" activeTab="7"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6930" firstSheet="4" activeTab="7"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12210"/>
   </bookViews>
   <sheets>
-    <sheet name="Primary cooking source" sheetId="1" r:id="rId1"/>
-    <sheet name="LPG subsidy" sheetId="2" r:id="rId2"/>
-    <sheet name="Subsidized cylinder count" sheetId="3" r:id="rId3"/>
-    <sheet name="Average consumption - PC 30 day" sheetId="4" r:id="rId4"/>
-    <sheet name="Average cylinders - HH 1 yr" sheetId="6" r:id="rId5"/>
-    <sheet name="PPAC vs HCES lpg consumption" sheetId="5" r:id="rId6"/>
-    <sheet name="Share LPG and firewood exp" sheetId="7" r:id="rId7"/>
+    <sheet name="Contents" sheetId="8" r:id="rId1"/>
+    <sheet name="Primary cooking source" sheetId="1" r:id="rId2"/>
+    <sheet name="LPG subsidy" sheetId="2" r:id="rId3"/>
+    <sheet name="Subsidized cylinder count" sheetId="3" r:id="rId4"/>
+    <sheet name="Average consumption - PC 30 day" sheetId="4" r:id="rId5"/>
+    <sheet name="Average cylinders - HH 1 yr" sheetId="6" r:id="rId6"/>
+    <sheet name="PPAC vs HCES lpg consumption" sheetId="5" r:id="rId7"/>
+    <sheet name="Share LPG and firewood exp" sheetId="7" r:id="rId8"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -31,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="820" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="838" uniqueCount="170">
   <si>
     <t>sample_size</t>
   </si>
@@ -509,6 +511,58 @@
   <si>
     <t>Across Urban Deciles - LPG or Firewood primary cooking fuel</t>
   </si>
+  <si>
+    <t>Sno</t>
+  </si>
+  <si>
+    <t>Sheet</t>
+  </si>
+  <si>
+    <t>Details</t>
+  </si>
+  <si>
+    <t>LPG subsidy</t>
+  </si>
+  <si>
+    <t>Subsidized cylinder count</t>
+  </si>
+  <si>
+    <t>Average consumption - PC 30 day</t>
+  </si>
+  <si>
+    <t>Average cylinders - HH 1 yr</t>
+  </si>
+  <si>
+    <t>PPAC vs HCES LPG consumption</t>
+  </si>
+  <si>
+    <t>Share LPG and firewood exp</t>
+  </si>
+  <si>
+    <t>Percentage breakdown of households based on primary fuel used for cooking</t>
+  </si>
+  <si>
+    <t>Percentage breakdown of households based on access to LPG subsidy.</t>
+  </si>
+  <si>
+    <t>Percentage breakdown of households based on the number of subsidised LPG cylinders consumed in the last 3 months.</t>
+  </si>
+  <si>
+    <t>Average per capita consumption of LPG and firewood in the last 30 days.</t>
+  </si>
+  <si>
+    <t>Average number of 14.2 kg cylinders consumed by households in the last 1 year.</t>
+  </si>
+  <si>
+    <t>Share of monthly per capita expenditure on firewood and LPG.</t>
+  </si>
+  <si>
+    <t>Comparison of LPG consumption from HCES and PPAC.</t>
+  </si>
+  <si>
+    <t>This workbook contains a comparative analysis of various aspects of LPG and firewood consumption in India, as covered in the Household Consumption Expenditure Surveys for 2022-23 and 2023-24. These statistics help identify population groups that need to be targeted for improving LPG penetration in the country. 
+For each of the themes mentioned below, statistics were generated at the following granularity: (a) All India, (b) Rural vs Urban areas, and (c) Deciles in Rural and Urban areas.</t>
+  </si>
 </sst>
 </file>
 
@@ -589,7 +643,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -611,6 +665,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1004,7 +1064,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="162">
+  <cellXfs count="169">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1271,6 +1331,9 @@
     <xf numFmtId="1" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1313,6 +1376,9 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1346,9 +1412,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1358,8 +1421,22 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1644,59 +1721,248 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB65"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="B2:M14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.81640625" style="13" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" style="8" customWidth="1"/>
-    <col min="3" max="3" width="10.81640625" style="8" customWidth="1"/>
-    <col min="4" max="4" width="10.7265625" style="8" customWidth="1"/>
-    <col min="5" max="8" width="8.81640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.453125" style="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="12" width="8.81640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.7265625" style="14" customWidth="1"/>
-    <col min="14" max="15" width="8.7265625" style="36" customWidth="1"/>
-    <col min="16" max="16" width="15.453125" style="36" customWidth="1"/>
-    <col min="17" max="17" width="13.81640625" style="36" customWidth="1"/>
-    <col min="18" max="28" width="8.7265625" style="36" customWidth="1"/>
-    <col min="29" max="16384" width="8.7265625" style="36" hidden="1"/>
+    <col min="1" max="2" width="9.140625" style="162"/>
+    <col min="3" max="3" width="30.85546875" style="162" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="40.42578125" style="162" customWidth="1"/>
+    <col min="5" max="10" width="9.140625" style="162"/>
+    <col min="11" max="11" width="9.28515625" style="162" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="162"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="31" customHeight="1" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="132" t="s">
+    <row r="2" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="166" t="s">
+        <v>169</v>
+      </c>
+      <c r="C2" s="166"/>
+      <c r="D2" s="166"/>
+      <c r="E2" s="166"/>
+      <c r="F2" s="166"/>
+      <c r="G2" s="166"/>
+      <c r="H2" s="166"/>
+      <c r="I2" s="166"/>
+      <c r="J2" s="166"/>
+      <c r="K2" s="166"/>
+      <c r="L2" s="166"/>
+      <c r="M2" s="166"/>
+    </row>
+    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B3" s="166"/>
+      <c r="C3" s="166"/>
+      <c r="D3" s="166"/>
+      <c r="E3" s="166"/>
+      <c r="F3" s="166"/>
+      <c r="G3" s="166"/>
+      <c r="H3" s="166"/>
+      <c r="I3" s="166"/>
+      <c r="J3" s="166"/>
+      <c r="K3" s="166"/>
+      <c r="L3" s="166"/>
+      <c r="M3" s="166"/>
+    </row>
+    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B4" s="166"/>
+      <c r="C4" s="166"/>
+      <c r="D4" s="166"/>
+      <c r="E4" s="166"/>
+      <c r="F4" s="166"/>
+      <c r="G4" s="166"/>
+      <c r="H4" s="166"/>
+      <c r="I4" s="166"/>
+      <c r="J4" s="166"/>
+      <c r="K4" s="166"/>
+      <c r="L4" s="166"/>
+      <c r="M4" s="166"/>
+    </row>
+    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B5" s="166"/>
+      <c r="C5" s="166"/>
+      <c r="D5" s="166"/>
+      <c r="E5" s="166"/>
+      <c r="F5" s="166"/>
+      <c r="G5" s="166"/>
+      <c r="H5" s="166"/>
+      <c r="I5" s="166"/>
+      <c r="J5" s="166"/>
+      <c r="K5" s="166"/>
+      <c r="L5" s="166"/>
+      <c r="M5" s="166"/>
+    </row>
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B6" s="167"/>
+      <c r="C6" s="167"/>
+      <c r="D6" s="167"/>
+      <c r="E6" s="167"/>
+      <c r="F6" s="167"/>
+      <c r="G6" s="167"/>
+      <c r="H6" s="167"/>
+      <c r="I6" s="167"/>
+      <c r="J6" s="167"/>
+      <c r="K6" s="167"/>
+    </row>
+    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B7" s="163" t="s">
+        <v>153</v>
+      </c>
+      <c r="C7" s="163" t="s">
+        <v>154</v>
+      </c>
+      <c r="D7" s="163" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="8" spans="2:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="B8" s="164">
+        <v>1</v>
+      </c>
+      <c r="C8" s="168" t="s">
+        <v>142</v>
+      </c>
+      <c r="D8" s="165" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="9" spans="2:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="B9" s="164">
+        <v>2</v>
+      </c>
+      <c r="C9" s="168" t="s">
+        <v>156</v>
+      </c>
+      <c r="D9" s="165" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="10" spans="2:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="B10" s="164">
+        <v>3</v>
+      </c>
+      <c r="C10" s="168" t="s">
+        <v>157</v>
+      </c>
+      <c r="D10" s="165" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="11" spans="2:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="B11" s="164">
+        <v>4</v>
+      </c>
+      <c r="C11" s="168" t="s">
+        <v>158</v>
+      </c>
+      <c r="D11" s="165" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="12" spans="2:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="B12" s="164">
+        <v>5</v>
+      </c>
+      <c r="C12" s="168" t="s">
+        <v>159</v>
+      </c>
+      <c r="D12" s="165" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="13" spans="2:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="B13" s="164">
+        <v>6</v>
+      </c>
+      <c r="C13" s="168" t="s">
+        <v>160</v>
+      </c>
+      <c r="D13" s="165" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="14" spans="2:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="B14" s="164">
+        <v>7</v>
+      </c>
+      <c r="C14" s="168" t="s">
+        <v>161</v>
+      </c>
+      <c r="D14" s="165" t="s">
+        <v>167</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:M5"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C8" location="'Primary cooking source'!A1" display="Primary cooking source"/>
+    <hyperlink ref="C9" location="'LPG subsidy'!A1" display="LPG subsidy"/>
+    <hyperlink ref="C10" location="'Subsidized cylinder count'!A1" display="Subsidized cylinder count"/>
+    <hyperlink ref="C11" location="'Average consumption - PC 30 day'!A1" display="Average consumption - PC 30 day"/>
+    <hyperlink ref="C12" location="'Average cylinders - HH 1 yr'!A1" display="Average cylinders - HH 1 yr"/>
+    <hyperlink ref="C13" location="'PPAC vs HCES lpg consumption'!A1" display="PPAC vs HCES LPG consumption"/>
+    <hyperlink ref="C14" location="'Share LPG and firewood exp'!A1" display="Share LPG and firewood exp"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AB65"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.85546875" style="13" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" style="8" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" style="8" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" style="8" customWidth="1"/>
+    <col min="5" max="8" width="8.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="12" width="8.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.7109375" style="14" customWidth="1"/>
+    <col min="14" max="15" width="8.7109375" style="36" customWidth="1"/>
+    <col min="16" max="16" width="15.42578125" style="36" customWidth="1"/>
+    <col min="17" max="17" width="13.85546875" style="36" customWidth="1"/>
+    <col min="18" max="28" width="8.7109375" style="36" customWidth="1"/>
+    <col min="29" max="16384" width="8.7109375" style="36" hidden="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:28" ht="30.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="133" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="133"/>
-      <c r="C1" s="133"/>
-      <c r="D1" s="133"/>
-      <c r="E1" s="133"/>
-      <c r="F1" s="133"/>
-      <c r="G1" s="133"/>
-      <c r="H1" s="133"/>
-      <c r="I1" s="133"/>
-      <c r="J1" s="133"/>
-      <c r="K1" s="133"/>
-      <c r="L1" s="133"/>
-      <c r="M1" s="134"/>
-      <c r="N1" s="135" t="s">
+      <c r="B1" s="134"/>
+      <c r="C1" s="134"/>
+      <c r="D1" s="134"/>
+      <c r="E1" s="134"/>
+      <c r="F1" s="134"/>
+      <c r="G1" s="134"/>
+      <c r="H1" s="134"/>
+      <c r="I1" s="134"/>
+      <c r="J1" s="134"/>
+      <c r="K1" s="134"/>
+      <c r="L1" s="134"/>
+      <c r="M1" s="135"/>
+      <c r="N1" s="136" t="s">
         <v>50</v>
       </c>
-      <c r="O1" s="136"/>
-      <c r="P1" s="136"/>
-      <c r="Q1" s="136"/>
-      <c r="R1" s="136"/>
-      <c r="S1" s="136"/>
-      <c r="T1" s="136"/>
-      <c r="U1" s="136"/>
-      <c r="V1" s="136"/>
-      <c r="W1" s="136"/>
-      <c r="X1" s="136"/>
-      <c r="Y1" s="136"/>
-      <c r="Z1" s="136"/>
+      <c r="O1" s="137"/>
+      <c r="P1" s="137"/>
+      <c r="Q1" s="137"/>
+      <c r="R1" s="137"/>
+      <c r="S1" s="137"/>
+      <c r="T1" s="137"/>
+      <c r="U1" s="137"/>
+      <c r="V1" s="137"/>
+      <c r="W1" s="137"/>
+      <c r="X1" s="137"/>
+      <c r="Y1" s="137"/>
+      <c r="Z1" s="137"/>
       <c r="AA1" s="50"/>
       <c r="AB1" s="51"/>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
         <v>13</v>
       </c>
@@ -1704,7 +1970,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
         <v>30</v>
       </c>
@@ -1719,7 +1985,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
         <v>1</v>
       </c>
@@ -1735,7 +2001,7 @@
       </c>
       <c r="X6" s="40"/>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
         <v>2</v>
       </c>
@@ -1751,7 +2017,7 @@
       </c>
       <c r="X7" s="40"/>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
         <v>3</v>
       </c>
@@ -1767,7 +2033,7 @@
       </c>
       <c r="X8" s="40"/>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
         <v>4</v>
       </c>
@@ -1783,7 +2049,7 @@
       </c>
       <c r="X9" s="40"/>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
         <v>5</v>
       </c>
@@ -1799,7 +2065,7 @@
       </c>
       <c r="X10" s="40"/>
     </row>
-    <row r="11" spans="1:28" ht="26" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:28" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
         <v>6</v>
       </c>
@@ -1815,7 +2081,7 @@
       </c>
       <c r="X11" s="40"/>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
         <v>7</v>
       </c>
@@ -1831,7 +2097,7 @@
       </c>
       <c r="X12" s="40"/>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
         <v>8</v>
       </c>
@@ -1847,7 +2113,7 @@
       </c>
       <c r="X13" s="40"/>
     </row>
-    <row r="14" spans="1:28" ht="26" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:28" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
         <v>9</v>
       </c>
@@ -1863,7 +2129,7 @@
       </c>
       <c r="X14" s="40"/>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
         <v>10</v>
       </c>
@@ -1879,7 +2145,7 @@
       </c>
       <c r="X15" s="40"/>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
         <v>11</v>
       </c>
@@ -1895,7 +2161,7 @@
       </c>
       <c r="X16" s="40"/>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
         <v>12</v>
       </c>
@@ -1911,7 +2177,7 @@
       </c>
       <c r="X17" s="40"/>
     </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
         <v>18</v>
       </c>
@@ -1921,7 +2187,7 @@
       <c r="Q20" s="42"/>
       <c r="R20" s="42"/>
     </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
         <v>30</v>
       </c>
@@ -1947,7 +2213,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
         <v>1</v>
       </c>
@@ -1973,7 +2239,7 @@
         <v>0.83705611874626162</v>
       </c>
     </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
         <v>2</v>
       </c>
@@ -1999,7 +2265,7 @@
         <v>1.8568948013527524E-4</v>
       </c>
     </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A24" s="18" t="s">
         <v>3</v>
       </c>
@@ -2025,7 +2291,7 @@
         <v>3.7733444560950169E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
         <v>4</v>
       </c>
@@ -2051,7 +2317,7 @@
         <v>1.6119084176994987E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A26" s="18" t="s">
         <v>5</v>
       </c>
@@ -2077,7 +2343,7 @@
         <v>1.6479223061002025E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A27" s="18" t="s">
         <v>6</v>
       </c>
@@ -2103,7 +2369,7 @@
         <v>4.7201383753768845E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A28" s="18" t="s">
         <v>7</v>
       </c>
@@ -2129,7 +2395,7 @@
         <v>4.3387372708699213E-5</v>
       </c>
     </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A29" s="18" t="s">
         <v>8</v>
       </c>
@@ -2155,7 +2421,7 @@
         <v>9.8264363919007484E-4</v>
       </c>
     </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A30" s="18" t="s">
         <v>9</v>
       </c>
@@ -2181,7 +2447,7 @@
         <v>6.8090249448486351E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A31" s="18" t="s">
         <v>10</v>
       </c>
@@ -2207,7 +2473,7 @@
         <v>2.221014796842432E-5</v>
       </c>
     </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A32" s="18" t="s">
         <v>11</v>
       </c>
@@ -2233,7 +2499,7 @@
         <v>3.6380556532290831E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A33" s="18" t="s">
         <v>12</v>
       </c>
@@ -2259,7 +2525,7 @@
         <v>3.0045856992951432E-3</v>
       </c>
     </row>
-    <row r="36" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
         <v>19</v>
       </c>
@@ -2267,7 +2533,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="37" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A37" s="16" t="s">
         <v>30</v>
       </c>
@@ -2335,7 +2601,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="38" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A38" s="19" t="s">
         <v>1</v>
       </c>
@@ -2403,7 +2669,7 @@
         <v>0.75907752972056086</v>
       </c>
     </row>
-    <row r="39" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A39" s="19" t="s">
         <v>2</v>
       </c>
@@ -2471,7 +2737,7 @@
         <v>4.4443758563725981E-5</v>
       </c>
     </row>
-    <row r="40" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A40" s="19" t="s">
         <v>3</v>
       </c>
@@ -2539,7 +2805,7 @@
         <v>6.9980533615526959E-4</v>
       </c>
     </row>
-    <row r="41" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A41" s="19" t="s">
         <v>4</v>
       </c>
@@ -2607,7 +2873,7 @@
         <v>4.9390700578847068E-3</v>
       </c>
     </row>
-    <row r="42" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A42" s="19" t="s">
         <v>5</v>
       </c>
@@ -2675,7 +2941,7 @@
         <v>3.4460013954975745E-3</v>
       </c>
     </row>
-    <row r="43" spans="1:26" ht="26" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:26" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A43" s="19" t="s">
         <v>6</v>
       </c>
@@ -2743,7 +3009,7 @@
         <v>0.20008977347675902</v>
       </c>
     </row>
-    <row r="44" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A44" s="19" t="s">
         <v>7</v>
       </c>
@@ -2811,7 +3077,7 @@
         <v>6.1559252252184728E-4</v>
       </c>
     </row>
-    <row r="45" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A45" s="19" t="s">
         <v>8</v>
       </c>
@@ -2879,7 +3145,7 @@
         <v>2.0826757082947046E-4</v>
       </c>
     </row>
-    <row r="46" spans="1:26" ht="26" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:26" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A46" s="19" t="s">
         <v>9</v>
       </c>
@@ -2947,7 +3213,7 @@
         <v>2.1648917416643248E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A47" s="19" t="s">
         <v>10</v>
       </c>
@@ -3015,7 +3281,7 @@
         <v>1.6654291749447722E-4</v>
       </c>
     </row>
-    <row r="48" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A48" s="19" t="s">
         <v>11</v>
       </c>
@@ -3083,7 +3349,7 @@
         <v>4.4428379091717863E-3</v>
       </c>
     </row>
-    <row r="49" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A49" s="19" t="s">
         <v>12</v>
       </c>
@@ -3151,7 +3417,7 @@
         <v>4.621217917918005E-3</v>
       </c>
     </row>
-    <row r="52" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A52" s="15" t="s">
         <v>20</v>
       </c>
@@ -3169,7 +3435,7 @@
       <c r="Y52" s="47"/>
       <c r="Z52" s="47"/>
     </row>
-    <row r="53" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A53" s="16" t="s">
         <v>30</v>
       </c>
@@ -3237,7 +3503,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="54" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A54" s="19" t="s">
         <v>1</v>
       </c>
@@ -3305,7 +3571,7 @@
         <v>0.66757494488783664</v>
       </c>
     </row>
-    <row r="55" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A55" s="19" t="s">
         <v>2</v>
       </c>
@@ -3373,7 +3639,7 @@
         <v>4.05045156051535E-5</v>
       </c>
     </row>
-    <row r="56" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A56" s="19" t="s">
         <v>3</v>
       </c>
@@ -3441,7 +3707,7 @@
         <v>1.0707338087731108E-5</v>
       </c>
     </row>
-    <row r="57" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A57" s="19" t="s">
         <v>4</v>
       </c>
@@ -3509,7 +3775,7 @@
         <v>3.1244925104173192E-5</v>
       </c>
     </row>
-    <row r="58" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A58" s="19" t="s">
         <v>5</v>
       </c>
@@ -3577,7 +3843,7 @@
         <v>4.6731720190177324E-3</v>
       </c>
     </row>
-    <row r="59" spans="1:26" ht="26" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:26" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A59" s="19" t="s">
         <v>6</v>
       </c>
@@ -3645,7 +3911,7 @@
         <v>5.4845473829500217E-3</v>
       </c>
     </row>
-    <row r="60" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A60" s="19" t="s">
         <v>7</v>
       </c>
@@ -3713,7 +3979,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A61" s="19" t="s">
         <v>8</v>
       </c>
@@ -3781,7 +4047,7 @@
         <v>3.278350096157566E-4</v>
       </c>
     </row>
-    <row r="62" spans="1:26" ht="26" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:26" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A62" s="19" t="s">
         <v>9</v>
       </c>
@@ -3849,7 +4115,7 @@
         <v>0.23720625534043091</v>
       </c>
     </row>
-    <row r="63" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A63" s="19" t="s">
         <v>10</v>
       </c>
@@ -3917,7 +4183,7 @@
         <v>1.2891681542130404E-4</v>
       </c>
     </row>
-    <row r="64" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A64" s="19" t="s">
         <v>11</v>
       </c>
@@ -3985,7 +4251,7 @@
         <v>8.024466696900473E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A65" s="19" t="s">
         <v>12</v>
       </c>
@@ -4063,63 +4329,63 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AD25"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.7265625" style="13" customWidth="1"/>
-    <col min="2" max="2" width="17.7265625" style="8" customWidth="1"/>
-    <col min="3" max="3" width="10.1796875" style="8" customWidth="1"/>
-    <col min="4" max="4" width="10.36328125" style="8" customWidth="1"/>
-    <col min="5" max="5" width="11.26953125" style="8" customWidth="1"/>
-    <col min="6" max="13" width="8.7265625" style="8" customWidth="1"/>
-    <col min="14" max="14" width="8.7265625" style="14" customWidth="1"/>
-    <col min="15" max="16" width="8.7265625" style="36" customWidth="1"/>
-    <col min="17" max="17" width="19.36328125" style="36" customWidth="1"/>
-    <col min="18" max="18" width="16.7265625" style="36" customWidth="1"/>
-    <col min="19" max="20" width="10.90625" style="36" customWidth="1"/>
-    <col min="21" max="30" width="8.7265625" style="36" customWidth="1"/>
-    <col min="31" max="16384" width="8.7265625" style="36" hidden="1"/>
+    <col min="1" max="1" width="19.7109375" style="13" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" style="8" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" style="8" customWidth="1"/>
+    <col min="4" max="4" width="10.42578125" style="8" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" style="8" customWidth="1"/>
+    <col min="6" max="13" width="8.7109375" style="8" customWidth="1"/>
+    <col min="14" max="14" width="8.7109375" style="14" customWidth="1"/>
+    <col min="15" max="16" width="8.7109375" style="36" customWidth="1"/>
+    <col min="17" max="17" width="19.42578125" style="36" customWidth="1"/>
+    <col min="18" max="18" width="16.7109375" style="36" customWidth="1"/>
+    <col min="19" max="20" width="10.85546875" style="36" customWidth="1"/>
+    <col min="21" max="30" width="8.7109375" style="36" customWidth="1"/>
+    <col min="31" max="16384" width="8.7109375" style="36" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="137" t="s">
+    <row r="1" spans="1:30" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="138" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="138"/>
-      <c r="C1" s="138"/>
-      <c r="D1" s="138"/>
-      <c r="E1" s="138"/>
-      <c r="F1" s="138"/>
-      <c r="G1" s="138"/>
-      <c r="H1" s="138"/>
-      <c r="I1" s="138"/>
-      <c r="J1" s="138"/>
-      <c r="K1" s="138"/>
-      <c r="L1" s="138"/>
-      <c r="M1" s="138"/>
-      <c r="N1" s="138"/>
-      <c r="O1" s="135" t="s">
+      <c r="B1" s="139"/>
+      <c r="C1" s="139"/>
+      <c r="D1" s="139"/>
+      <c r="E1" s="139"/>
+      <c r="F1" s="139"/>
+      <c r="G1" s="139"/>
+      <c r="H1" s="139"/>
+      <c r="I1" s="139"/>
+      <c r="J1" s="139"/>
+      <c r="K1" s="139"/>
+      <c r="L1" s="139"/>
+      <c r="M1" s="139"/>
+      <c r="N1" s="139"/>
+      <c r="O1" s="136" t="s">
         <v>50</v>
       </c>
-      <c r="P1" s="136"/>
-      <c r="Q1" s="136"/>
-      <c r="R1" s="136"/>
-      <c r="S1" s="136"/>
-      <c r="T1" s="136"/>
-      <c r="U1" s="136"/>
-      <c r="V1" s="136"/>
-      <c r="W1" s="136"/>
-      <c r="X1" s="136"/>
-      <c r="Y1" s="136"/>
-      <c r="Z1" s="136"/>
-      <c r="AA1" s="136"/>
-      <c r="AB1" s="136"/>
+      <c r="P1" s="137"/>
+      <c r="Q1" s="137"/>
+      <c r="R1" s="137"/>
+      <c r="S1" s="137"/>
+      <c r="T1" s="137"/>
+      <c r="U1" s="137"/>
+      <c r="V1" s="137"/>
+      <c r="W1" s="137"/>
+      <c r="X1" s="137"/>
+      <c r="Y1" s="137"/>
+      <c r="Z1" s="137"/>
+      <c r="AA1" s="137"/>
+      <c r="AB1" s="137"/>
       <c r="AC1" s="50"/>
       <c r="AD1" s="51"/>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
         <v>38</v>
       </c>
@@ -4130,7 +4396,7 @@
       <c r="S4" s="42"/>
       <c r="T4" s="42"/>
     </row>
-    <row r="5" spans="1:30" ht="34" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:30" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="24" t="s">
         <v>21</v>
       </c>
@@ -4156,7 +4422,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:30" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="25" t="s">
         <v>22</v>
       </c>
@@ -4184,7 +4450,7 @@
         <v>0.70195876001560165</v>
       </c>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
         <v>23</v>
       </c>
@@ -4212,7 +4478,7 @@
         <v>0.29804123998439841</v>
       </c>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
         <v>35</v>
       </c>
@@ -4220,7 +4486,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="26" t="s">
         <v>26</v>
       </c>
@@ -4240,7 +4506,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:30" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
         <v>22</v>
       </c>
@@ -4262,7 +4528,7 @@
       <c r="T12" s="40"/>
       <c r="U12" s="40"/>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
         <v>23</v>
       </c>
@@ -4284,7 +4550,7 @@
       <c r="T13" s="40"/>
       <c r="U13" s="40"/>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
         <v>39</v>
       </c>
@@ -4303,7 +4569,7 @@
       <c r="AA16" s="47"/>
       <c r="AB16" s="47"/>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
         <v>27</v>
       </c>
@@ -4377,7 +4643,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:28" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="28" t="s">
         <v>24</v>
       </c>
@@ -4451,7 +4717,7 @@
         <v>0.64611687037606713</v>
       </c>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
         <v>24</v>
       </c>
@@ -4525,7 +4791,7 @@
         <v>0.35388312962393287</v>
       </c>
     </row>
-    <row r="20" spans="1:28" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="18" t="s">
         <v>25</v>
       </c>
@@ -4599,7 +4865,7 @@
         <v>0.86479574314550922</v>
       </c>
     </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
         <v>25</v>
       </c>
@@ -4673,7 +4939,7 @@
         <v>0.13520425685449078</v>
       </c>
     </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
       <c r="S22" s="40"/>
       <c r="T22" s="40"/>
       <c r="U22" s="40"/>
@@ -4685,7 +4951,7 @@
       <c r="AA22" s="40"/>
       <c r="AB22" s="40"/>
     </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
       <c r="S23" s="40"/>
       <c r="T23" s="40"/>
       <c r="U23" s="40"/>
@@ -4697,7 +4963,7 @@
       <c r="AA23" s="40"/>
       <c r="AB23" s="40"/>
     </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
       <c r="S24" s="40"/>
       <c r="T24" s="40"/>
       <c r="U24" s="40"/>
@@ -4709,7 +4975,7 @@
       <c r="AA24" s="40"/>
       <c r="AB24" s="40"/>
     </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
       <c r="S25" s="40"/>
       <c r="T25" s="40"/>
       <c r="U25" s="40"/>
@@ -4730,58 +4996,58 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AB31"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.08984375" style="13" customWidth="1"/>
+    <col min="1" max="1" width="10.140625" style="13" customWidth="1"/>
     <col min="2" max="2" width="11" style="8" customWidth="1"/>
-    <col min="3" max="12" width="8.7265625" style="8" customWidth="1"/>
-    <col min="13" max="13" width="8.7265625" style="14" customWidth="1"/>
-    <col min="14" max="14" width="8.7265625" style="54" customWidth="1"/>
-    <col min="15" max="15" width="8.7265625" style="42" customWidth="1"/>
-    <col min="16" max="16" width="10.7265625" style="42" customWidth="1"/>
-    <col min="17" max="27" width="8.7265625" style="42" customWidth="1"/>
-    <col min="28" max="28" width="8.7265625" style="55" customWidth="1"/>
-    <col min="29" max="16384" width="8.7265625" hidden="1"/>
+    <col min="3" max="12" width="8.7109375" style="8" customWidth="1"/>
+    <col min="13" max="13" width="8.7109375" style="14" customWidth="1"/>
+    <col min="14" max="14" width="8.7109375" style="54" customWidth="1"/>
+    <col min="15" max="15" width="8.7109375" style="42" customWidth="1"/>
+    <col min="16" max="16" width="10.7109375" style="42" customWidth="1"/>
+    <col min="17" max="27" width="8.7109375" style="42" customWidth="1"/>
+    <col min="28" max="28" width="8.7109375" style="55" customWidth="1"/>
+    <col min="29" max="16384" width="8.7109375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="29" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="137" t="s">
+    <row r="1" spans="1:28" ht="29.25" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="138" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="138"/>
-      <c r="C1" s="138"/>
-      <c r="D1" s="138"/>
-      <c r="E1" s="138"/>
-      <c r="F1" s="138"/>
-      <c r="G1" s="138"/>
-      <c r="H1" s="138"/>
-      <c r="I1" s="138"/>
-      <c r="J1" s="138"/>
-      <c r="K1" s="138"/>
-      <c r="L1" s="138"/>
-      <c r="M1" s="141"/>
-      <c r="N1" s="135" t="s">
+      <c r="B1" s="139"/>
+      <c r="C1" s="139"/>
+      <c r="D1" s="139"/>
+      <c r="E1" s="139"/>
+      <c r="F1" s="139"/>
+      <c r="G1" s="139"/>
+      <c r="H1" s="139"/>
+      <c r="I1" s="139"/>
+      <c r="J1" s="139"/>
+      <c r="K1" s="139"/>
+      <c r="L1" s="139"/>
+      <c r="M1" s="142"/>
+      <c r="N1" s="136" t="s">
         <v>49</v>
       </c>
-      <c r="O1" s="136"/>
-      <c r="P1" s="136"/>
-      <c r="Q1" s="136"/>
-      <c r="R1" s="136"/>
-      <c r="S1" s="136"/>
-      <c r="T1" s="136"/>
-      <c r="U1" s="136"/>
-      <c r="V1" s="136"/>
-      <c r="W1" s="136"/>
-      <c r="X1" s="136"/>
-      <c r="Y1" s="136"/>
-      <c r="Z1" s="136"/>
-      <c r="AA1" s="136"/>
-      <c r="AB1" s="139"/>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="O1" s="137"/>
+      <c r="P1" s="137"/>
+      <c r="Q1" s="137"/>
+      <c r="R1" s="137"/>
+      <c r="S1" s="137"/>
+      <c r="T1" s="137"/>
+      <c r="U1" s="137"/>
+      <c r="V1" s="137"/>
+      <c r="W1" s="137"/>
+      <c r="X1" s="137"/>
+      <c r="Y1" s="137"/>
+      <c r="Z1" s="137"/>
+      <c r="AA1" s="137"/>
+      <c r="AB1" s="140"/>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
         <v>34</v>
       </c>
@@ -4789,7 +5055,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="26" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:28" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="26" t="s">
         <v>29</v>
       </c>
@@ -4815,7 +5081,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" s="32">
         <v>1</v>
       </c>
@@ -4843,7 +5109,7 @@
         <v>0.5816338165459064</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" s="32">
         <v>2</v>
       </c>
@@ -4871,7 +5137,7 @@
         <v>0.30053775568593571</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" s="32">
         <v>3</v>
       </c>
@@ -4899,7 +5165,7 @@
         <v>0.1178284277681579</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
         <v>35</v>
       </c>
@@ -4907,7 +5173,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:28" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="33" t="s">
         <v>29</v>
       </c>
@@ -4927,7 +5193,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" s="24">
         <v>1</v>
       </c>
@@ -4947,7 +5213,7 @@
         <v>0.47193796123272519</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" s="24">
         <v>2</v>
       </c>
@@ -4967,7 +5233,7 @@
         <v>0.36810750040269202</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" s="24">
         <v>3</v>
       </c>
@@ -4987,7 +5253,7 @@
         <v>0.15995453836458282</v>
       </c>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
         <v>36</v>
       </c>
@@ -5005,40 +5271,40 @@
       <c r="Y18" s="41"/>
       <c r="Z18" s="41"/>
     </row>
-    <row r="19" spans="1:26" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="142" t="s">
+    <row r="19" spans="1:26" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="143" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="140" t="s">
+      <c r="B19" s="141" t="s">
         <v>48</v>
       </c>
-      <c r="C19" s="140"/>
-      <c r="D19" s="140"/>
-      <c r="E19" s="140"/>
-      <c r="F19" s="140"/>
-      <c r="G19" s="140"/>
-      <c r="H19" s="140"/>
-      <c r="I19" s="140"/>
-      <c r="J19" s="140"/>
-      <c r="K19" s="140"/>
-      <c r="P19" s="145" t="s">
+      <c r="C19" s="141"/>
+      <c r="D19" s="141"/>
+      <c r="E19" s="141"/>
+      <c r="F19" s="141"/>
+      <c r="G19" s="141"/>
+      <c r="H19" s="141"/>
+      <c r="I19" s="141"/>
+      <c r="J19" s="141"/>
+      <c r="K19" s="141"/>
+      <c r="P19" s="146" t="s">
         <v>29</v>
       </c>
-      <c r="Q19" s="144" t="s">
+      <c r="Q19" s="145" t="s">
         <v>48</v>
       </c>
-      <c r="R19" s="144"/>
-      <c r="S19" s="144"/>
-      <c r="T19" s="144"/>
-      <c r="U19" s="144"/>
-      <c r="V19" s="144"/>
-      <c r="W19" s="144"/>
-      <c r="X19" s="144"/>
-      <c r="Y19" s="144"/>
-      <c r="Z19" s="144"/>
-    </row>
-    <row r="20" spans="1:26" ht="13" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="143"/>
+      <c r="R19" s="145"/>
+      <c r="S19" s="145"/>
+      <c r="T19" s="145"/>
+      <c r="U19" s="145"/>
+      <c r="V19" s="145"/>
+      <c r="W19" s="145"/>
+      <c r="X19" s="145"/>
+      <c r="Y19" s="145"/>
+      <c r="Z19" s="145"/>
+    </row>
+    <row r="20" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="144"/>
       <c r="B20" s="2">
         <v>1</v>
       </c>
@@ -5069,7 +5335,7 @@
       <c r="K20" s="2">
         <v>10</v>
       </c>
-      <c r="P20" s="145"/>
+      <c r="P20" s="146"/>
       <c r="Q20" s="43">
         <v>1</v>
       </c>
@@ -5101,7 +5367,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A21" s="24">
         <v>1</v>
       </c>
@@ -5169,7 +5435,7 @@
         <v>0.60584838770470795</v>
       </c>
     </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A22" s="24">
         <v>2</v>
       </c>
@@ -5237,7 +5503,7 @@
         <v>0.29179413104353347</v>
       </c>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A23" s="24">
         <v>3</v>
       </c>
@@ -5305,7 +5571,7 @@
         <v>0.10235748125175866</v>
       </c>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
         <v>37</v>
       </c>
@@ -5323,40 +5589,40 @@
       <c r="Y26" s="41"/>
       <c r="Z26" s="41"/>
     </row>
-    <row r="27" spans="1:26" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="142" t="s">
+    <row r="27" spans="1:26" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="143" t="s">
         <v>29</v>
       </c>
-      <c r="B27" s="140" t="s">
+      <c r="B27" s="141" t="s">
         <v>48</v>
       </c>
-      <c r="C27" s="140"/>
-      <c r="D27" s="140"/>
-      <c r="E27" s="140"/>
-      <c r="F27" s="140"/>
-      <c r="G27" s="140"/>
-      <c r="H27" s="140"/>
-      <c r="I27" s="140"/>
-      <c r="J27" s="140"/>
-      <c r="K27" s="140"/>
-      <c r="P27" s="145" t="s">
+      <c r="C27" s="141"/>
+      <c r="D27" s="141"/>
+      <c r="E27" s="141"/>
+      <c r="F27" s="141"/>
+      <c r="G27" s="141"/>
+      <c r="H27" s="141"/>
+      <c r="I27" s="141"/>
+      <c r="J27" s="141"/>
+      <c r="K27" s="141"/>
+      <c r="P27" s="146" t="s">
         <v>29</v>
       </c>
-      <c r="Q27" s="144" t="s">
+      <c r="Q27" s="145" t="s">
         <v>48</v>
       </c>
-      <c r="R27" s="144"/>
-      <c r="S27" s="144"/>
-      <c r="T27" s="144"/>
-      <c r="U27" s="144"/>
-      <c r="V27" s="144"/>
-      <c r="W27" s="144"/>
-      <c r="X27" s="144"/>
-      <c r="Y27" s="144"/>
-      <c r="Z27" s="144"/>
-    </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A28" s="143"/>
+      <c r="R27" s="145"/>
+      <c r="S27" s="145"/>
+      <c r="T27" s="145"/>
+      <c r="U27" s="145"/>
+      <c r="V27" s="145"/>
+      <c r="W27" s="145"/>
+      <c r="X27" s="145"/>
+      <c r="Y27" s="145"/>
+      <c r="Z27" s="145"/>
+    </row>
+    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A28" s="144"/>
       <c r="B28" s="2">
         <v>1</v>
       </c>
@@ -5387,7 +5653,7 @@
       <c r="K28" s="2">
         <v>10</v>
       </c>
-      <c r="P28" s="145"/>
+      <c r="P28" s="146"/>
       <c r="Q28" s="43">
         <v>1</v>
       </c>
@@ -5419,7 +5685,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A29" s="24">
         <v>1</v>
       </c>
@@ -5487,7 +5753,7 @@
         <v>0.4810634587675417</v>
       </c>
     </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A30" s="24">
         <v>2</v>
       </c>
@@ -5555,7 +5821,7 @@
         <v>0.36962414885104078</v>
       </c>
     </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A31" s="24">
         <v>3</v>
       </c>
@@ -5640,69 +5906,69 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AE195"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.54296875" style="13" customWidth="1"/>
-    <col min="2" max="6" width="12.26953125" style="8" customWidth="1"/>
-    <col min="7" max="7" width="13.08984375" style="8" customWidth="1"/>
-    <col min="8" max="8" width="20.26953125" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.26953125" style="8" customWidth="1"/>
-    <col min="10" max="11" width="13.08984375" style="8" customWidth="1"/>
-    <col min="12" max="14" width="8.7265625" style="8" customWidth="1"/>
-    <col min="15" max="15" width="8.7265625" style="14" customWidth="1"/>
-    <col min="16" max="16" width="8.7265625" style="54" customWidth="1"/>
-    <col min="17" max="17" width="8.7265625" style="42" customWidth="1"/>
-    <col min="18" max="18" width="22.1796875" style="42" customWidth="1"/>
-    <col min="19" max="24" width="12.26953125" style="42" customWidth="1"/>
-    <col min="25" max="25" width="20.26953125" style="42" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="14.26953125" style="42" customWidth="1"/>
-    <col min="27" max="28" width="12.90625" style="42" customWidth="1"/>
-    <col min="29" max="30" width="8.7265625" style="42" customWidth="1"/>
-    <col min="31" max="31" width="8.7265625" style="55" customWidth="1"/>
-    <col min="32" max="16384" width="8.7265625" hidden="1"/>
+    <col min="1" max="1" width="24.5703125" style="13" customWidth="1"/>
+    <col min="2" max="6" width="12.28515625" style="8" customWidth="1"/>
+    <col min="7" max="7" width="13.140625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="20.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.28515625" style="8" customWidth="1"/>
+    <col min="10" max="11" width="13.140625" style="8" customWidth="1"/>
+    <col min="12" max="14" width="8.7109375" style="8" customWidth="1"/>
+    <col min="15" max="15" width="8.7109375" style="14" customWidth="1"/>
+    <col min="16" max="16" width="8.7109375" style="54" customWidth="1"/>
+    <col min="17" max="17" width="8.7109375" style="42" customWidth="1"/>
+    <col min="18" max="18" width="22.140625" style="42" customWidth="1"/>
+    <col min="19" max="24" width="12.28515625" style="42" customWidth="1"/>
+    <col min="25" max="25" width="20.28515625" style="42" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="14.28515625" style="42" customWidth="1"/>
+    <col min="27" max="28" width="12.85546875" style="42" customWidth="1"/>
+    <col min="29" max="30" width="8.7109375" style="42" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" style="55" customWidth="1"/>
+    <col min="32" max="16384" width="8.7109375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="29" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="137" t="s">
+    <row r="1" spans="1:31" ht="29.25" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="138" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="138"/>
-      <c r="C1" s="138"/>
-      <c r="D1" s="138"/>
-      <c r="E1" s="138"/>
-      <c r="F1" s="138"/>
-      <c r="G1" s="138"/>
-      <c r="H1" s="138"/>
-      <c r="I1" s="138"/>
-      <c r="J1" s="138"/>
-      <c r="K1" s="138"/>
-      <c r="L1" s="138"/>
-      <c r="M1" s="138"/>
-      <c r="N1" s="138"/>
-      <c r="O1" s="141"/>
-      <c r="P1" s="135" t="s">
+      <c r="B1" s="139"/>
+      <c r="C1" s="139"/>
+      <c r="D1" s="139"/>
+      <c r="E1" s="139"/>
+      <c r="F1" s="139"/>
+      <c r="G1" s="139"/>
+      <c r="H1" s="139"/>
+      <c r="I1" s="139"/>
+      <c r="J1" s="139"/>
+      <c r="K1" s="139"/>
+      <c r="L1" s="139"/>
+      <c r="M1" s="139"/>
+      <c r="N1" s="139"/>
+      <c r="O1" s="142"/>
+      <c r="P1" s="136" t="s">
         <v>50</v>
       </c>
-      <c r="Q1" s="136"/>
-      <c r="R1" s="136"/>
-      <c r="S1" s="136"/>
-      <c r="T1" s="136"/>
-      <c r="U1" s="136"/>
-      <c r="V1" s="136"/>
-      <c r="W1" s="136"/>
-      <c r="X1" s="136"/>
-      <c r="Y1" s="136"/>
-      <c r="Z1" s="136"/>
-      <c r="AA1" s="136"/>
-      <c r="AB1" s="136"/>
-      <c r="AC1" s="136"/>
-      <c r="AD1" s="136"/>
-      <c r="AE1" s="139"/>
-    </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="Q1" s="137"/>
+      <c r="R1" s="137"/>
+      <c r="S1" s="137"/>
+      <c r="T1" s="137"/>
+      <c r="U1" s="137"/>
+      <c r="V1" s="137"/>
+      <c r="W1" s="137"/>
+      <c r="X1" s="137"/>
+      <c r="Y1" s="137"/>
+      <c r="Z1" s="137"/>
+      <c r="AA1" s="137"/>
+      <c r="AB1" s="137"/>
+      <c r="AC1" s="137"/>
+      <c r="AD1" s="137"/>
+      <c r="AE1" s="140"/>
+    </row>
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
         <v>40</v>
       </c>
@@ -5710,7 +5976,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
         <v>31</v>
       </c>
@@ -5730,7 +5996,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
         <v>45</v>
       </c>
@@ -5750,7 +6016,7 @@
         <v>1.5981240000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
         <v>46</v>
       </c>
@@ -5773,7 +6039,7 @@
         <v>106.07063599999999</v>
       </c>
     </row>
-    <row r="8" spans="1:31" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:31" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="69" t="s">
         <v>98</v>
       </c>
@@ -5802,7 +6068,7 @@
         <v>2.1273066869622577</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A9" s="18" t="s">
         <v>51</v>
       </c>
@@ -5831,7 +6097,7 @@
         <v>9.9373509999999996</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A10" s="18" t="s">
         <v>52</v>
       </c>
@@ -5862,7 +6128,7 @@
       </c>
       <c r="U10" s="64"/>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>53</v>
       </c>
@@ -5884,7 +6150,7 @@
       </c>
       <c r="U11" s="64"/>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>54</v>
       </c>
@@ -5909,7 +6175,7 @@
         <v>4.8522095112909644</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A13" s="99" t="s">
         <v>133</v>
       </c>
@@ -5933,7 +6199,7 @@
       </c>
       <c r="U13" s="64"/>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A14" s="99" t="s">
         <v>132</v>
       </c>
@@ -5957,7 +6223,7 @@
       </c>
       <c r="U14" s="64"/>
     </row>
-    <row r="15" spans="1:31" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:31" ht="36.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="69" t="s">
         <v>104</v>
       </c>
@@ -5981,13 +6247,13 @@
       </c>
       <c r="U15" s="64"/>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A16" s="15"/>
     </row>
-    <row r="17" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="15"/>
     </row>
-    <row r="18" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
         <v>42</v>
       </c>
@@ -5997,12 +6263,12 @@
       <c r="S18" s="41"/>
       <c r="T18" s="41"/>
     </row>
-    <row r="19" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="15"/>
-      <c r="C19" s="157" t="s">
+      <c r="C19" s="147" t="s">
         <v>41</v>
       </c>
-      <c r="D19" s="157"/>
+      <c r="D19" s="147"/>
       <c r="R19" s="41"/>
       <c r="S19" s="41"/>
       <c r="T19" s="41" t="s">
@@ -6012,7 +6278,7 @@
       <c r="AB19" s="36"/>
       <c r="AC19" s="36"/>
     </row>
-    <row r="20" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
         <v>31</v>
       </c>
@@ -6044,7 +6310,7 @@
       <c r="AB20" s="36"/>
       <c r="AC20" s="36"/>
     </row>
-    <row r="21" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
         <v>45</v>
       </c>
@@ -6076,7 +6342,7 @@
       <c r="AB21" s="36"/>
       <c r="AC21" s="36"/>
     </row>
-    <row r="22" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
         <v>46</v>
       </c>
@@ -6108,7 +6374,7 @@
       <c r="AB22" s="36"/>
       <c r="AC22" s="36"/>
     </row>
-    <row r="23" spans="1:29" ht="29" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:29" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="69" t="s">
         <v>98</v>
       </c>
@@ -6144,7 +6410,7 @@
       <c r="AB23" s="36"/>
       <c r="AC23" s="36"/>
     </row>
-    <row r="24" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="18" t="s">
         <v>51</v>
       </c>
@@ -6173,7 +6439,7 @@
         <v>2.0171420000000002</v>
       </c>
     </row>
-    <row r="25" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
         <v>52</v>
       </c>
@@ -6199,7 +6465,7 @@
         <v>10.07423</v>
       </c>
     </row>
-    <row r="26" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>53</v>
       </c>
@@ -6225,7 +6491,7 @@
         <v>1.574948</v>
       </c>
     </row>
-    <row r="27" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
         <v>54</v>
       </c>
@@ -6251,7 +6517,7 @@
         <v>8.4387450000000008</v>
       </c>
     </row>
-    <row r="28" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A28" s="99" t="s">
         <v>133</v>
       </c>
@@ -6281,7 +6547,7 @@
         <v>0.78078191817928522</v>
       </c>
     </row>
-    <row r="29" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A29" s="99" t="s">
         <v>132</v>
       </c>
@@ -6311,7 +6577,7 @@
         <v>0.8376565752419789</v>
       </c>
     </row>
-    <row r="30" spans="1:29" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="69" t="s">
         <v>104</v>
       </c>
@@ -6341,7 +6607,7 @@
         <v>2.232545931675205</v>
       </c>
     </row>
-    <row r="33" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
         <v>43</v>
       </c>
@@ -6360,7 +6626,7 @@
       <c r="AB33" s="41"/>
       <c r="AC33" s="41"/>
     </row>
-    <row r="34" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A34" s="16" t="s">
         <v>31</v>
       </c>
@@ -6434,7 +6700,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A35" s="18" t="s">
         <v>45</v>
       </c>
@@ -6508,7 +6774,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="36" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A36" s="18" t="s">
         <v>46</v>
       </c>
@@ -6582,7 +6848,7 @@
         <v>160.36000000000001</v>
       </c>
     </row>
-    <row r="37" spans="1:29" ht="29" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:29" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="69" t="s">
         <v>98</v>
       </c>
@@ -6676,7 +6942,7 @@
         <v>2.1326736886902862</v>
       </c>
     </row>
-    <row r="38" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A38" s="18" t="s">
         <v>51</v>
       </c>
@@ -6750,7 +7016,7 @@
         <v>10.31</v>
       </c>
     </row>
-    <row r="39" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A39" s="18" t="s">
         <v>52</v>
       </c>
@@ -6824,7 +7090,7 @@
         <v>48.98</v>
       </c>
     </row>
-    <row r="40" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
         <v>53</v>
       </c>
@@ -6898,7 +7164,7 @@
         <v>5.9979139999999997</v>
       </c>
     </row>
-    <row r="41" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
         <v>54</v>
       </c>
@@ -6972,7 +7238,7 @@
         <v>30.213107000000001</v>
       </c>
     </row>
-    <row r="42" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A42" s="99" t="s">
         <v>133</v>
       </c>
@@ -7066,7 +7332,7 @@
         <v>0.58175693501454895</v>
       </c>
     </row>
-    <row r="43" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A43" s="99" t="s">
         <v>132</v>
       </c>
@@ -7160,7 +7426,7 @@
         <v>0.61684579420171504</v>
       </c>
     </row>
-    <row r="44" spans="1:29" ht="29" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A44" s="69" t="s">
         <v>104</v>
       </c>
@@ -7254,7 +7520,7 @@
         <v>2.0988621349578094</v>
       </c>
     </row>
-    <row r="47" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A47" s="15" t="s">
         <v>44</v>
       </c>
@@ -7262,7 +7528,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="48" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A48" s="16" t="s">
         <v>31</v>
       </c>
@@ -7336,7 +7602,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="49" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A49" s="18" t="s">
         <v>45</v>
       </c>
@@ -7410,7 +7676,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="50" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A50" s="18" t="s">
         <v>46</v>
       </c>
@@ -7484,7 +7750,7 @@
         <v>181.46</v>
       </c>
     </row>
-    <row r="51" spans="1:31" ht="29" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:31" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="69" t="s">
         <v>98</v>
       </c>
@@ -7578,7 +7844,7 @@
         <v>2.1226370952648321</v>
       </c>
     </row>
-    <row r="52" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A52" s="18" t="s">
         <v>51</v>
       </c>
@@ -7652,7 +7918,7 @@
         <v>0.61</v>
       </c>
     </row>
-    <row r="53" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A53" s="18" t="s">
         <v>52</v>
       </c>
@@ -7726,7 +7992,7 @@
         <v>3.2</v>
       </c>
     </row>
-    <row r="54" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A54" s="9" t="s">
         <v>53</v>
       </c>
@@ -7800,7 +8066,7 @@
         <v>0.36595</v>
       </c>
     </row>
-    <row r="55" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="s">
         <v>54</v>
       </c>
@@ -7874,7 +8140,7 @@
         <v>2.259185</v>
       </c>
     </row>
-    <row r="56" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A56" s="99" t="s">
         <v>133</v>
       </c>
@@ -7968,7 +8234,7 @@
         <v>0.59991803278688527</v>
       </c>
     </row>
-    <row r="57" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A57" s="99" t="s">
         <v>132</v>
       </c>
@@ -8062,7 +8328,7 @@
         <v>0.70599531249999992</v>
       </c>
     </row>
-    <row r="58" spans="1:31" ht="29" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:31" ht="45" x14ac:dyDescent="0.25">
       <c r="A58" s="69" t="s">
         <v>104</v>
       </c>
@@ -8156,7 +8422,7 @@
         <v>2.572283326501799</v>
       </c>
     </row>
-    <row r="61" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A61" s="15" t="s">
         <v>94</v>
       </c>
@@ -8172,68 +8438,68 @@
       <c r="W61" s="36"/>
       <c r="X61" s="36"/>
     </row>
-    <row r="62" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A62" s="140" t="s">
+    <row r="62" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A62" s="141" t="s">
         <v>24</v>
       </c>
-      <c r="B62" s="140"/>
-      <c r="C62" s="140"/>
-      <c r="D62" s="140"/>
-      <c r="E62" s="140"/>
-      <c r="F62" s="140"/>
-      <c r="G62" s="140"/>
-      <c r="H62" s="140"/>
-      <c r="I62" s="140"/>
-      <c r="J62" s="140"/>
-      <c r="K62" s="140"/>
+      <c r="B62" s="141"/>
+      <c r="C62" s="141"/>
+      <c r="D62" s="141"/>
+      <c r="E62" s="141"/>
+      <c r="F62" s="141"/>
+      <c r="G62" s="141"/>
+      <c r="H62" s="141"/>
+      <c r="I62" s="141"/>
+      <c r="J62" s="141"/>
+      <c r="K62" s="141"/>
       <c r="L62" s="1"/>
-      <c r="R62" s="144" t="s">
+      <c r="R62" s="145" t="s">
         <v>24</v>
       </c>
-      <c r="S62" s="144"/>
-      <c r="T62" s="144"/>
-      <c r="U62" s="144"/>
-      <c r="V62" s="144"/>
-      <c r="W62" s="144"/>
-      <c r="X62" s="144"/>
-      <c r="Y62" s="144"/>
-      <c r="Z62" s="144"/>
-      <c r="AA62" s="144"/>
-      <c r="AB62" s="144"/>
-    </row>
-    <row r="63" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="S62" s="145"/>
+      <c r="T62" s="145"/>
+      <c r="U62" s="145"/>
+      <c r="V62" s="145"/>
+      <c r="W62" s="145"/>
+      <c r="X62" s="145"/>
+      <c r="Y62" s="145"/>
+      <c r="Z62" s="145"/>
+      <c r="AA62" s="145"/>
+      <c r="AB62" s="145"/>
+    </row>
+    <row r="63" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A63" s="9"/>
-      <c r="B63" s="150" t="s">
+      <c r="B63" s="152" t="s">
         <v>55</v>
       </c>
-      <c r="C63" s="150"/>
-      <c r="D63" s="150"/>
-      <c r="E63" s="150"/>
-      <c r="F63" s="150"/>
-      <c r="G63" s="150"/>
-      <c r="H63" s="150"/>
-      <c r="I63" s="147" t="s">
+      <c r="C63" s="152"/>
+      <c r="D63" s="152"/>
+      <c r="E63" s="152"/>
+      <c r="F63" s="152"/>
+      <c r="G63" s="152"/>
+      <c r="H63" s="152"/>
+      <c r="I63" s="149" t="s">
         <v>1</v>
       </c>
-      <c r="J63" s="148"/>
-      <c r="K63" s="149"/>
+      <c r="J63" s="150"/>
+      <c r="K63" s="151"/>
       <c r="R63" s="45"/>
-      <c r="S63" s="145" t="s">
+      <c r="S63" s="146" t="s">
         <v>55</v>
       </c>
-      <c r="T63" s="145"/>
-      <c r="U63" s="145"/>
-      <c r="V63" s="145"/>
-      <c r="W63" s="145"/>
-      <c r="X63" s="145"/>
-      <c r="Y63" s="145"/>
+      <c r="T63" s="146"/>
+      <c r="U63" s="146"/>
+      <c r="V63" s="146"/>
+      <c r="W63" s="146"/>
+      <c r="X63" s="146"/>
+      <c r="Y63" s="146"/>
       <c r="Z63" s="103" t="s">
         <v>1</v>
       </c>
       <c r="AA63" s="103"/>
       <c r="AB63" s="103"/>
     </row>
-    <row r="64" spans="1:31" s="36" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:31" s="36" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>56</v>
       </c>
@@ -8314,7 +8580,7 @@
       <c r="AD64" s="42"/>
       <c r="AE64" s="55"/>
     </row>
-    <row r="65" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="23" t="s">
         <v>57</v>
       </c>
@@ -8405,7 +8671,7 @@
       <c r="AD65" s="42"/>
       <c r="AE65" s="55"/>
     </row>
-    <row r="66" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="23" t="s">
         <v>58</v>
       </c>
@@ -8496,7 +8762,7 @@
       <c r="AD66" s="42"/>
       <c r="AE66" s="55"/>
     </row>
-    <row r="67" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="23" t="s">
         <v>59</v>
       </c>
@@ -8587,7 +8853,7 @@
       <c r="AD67" s="42"/>
       <c r="AE67" s="55"/>
     </row>
-    <row r="68" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="23" t="s">
         <v>60</v>
       </c>
@@ -8678,7 +8944,7 @@
       <c r="AD68" s="42"/>
       <c r="AE68" s="55"/>
     </row>
-    <row r="69" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="23" t="s">
         <v>61</v>
       </c>
@@ -8769,7 +9035,7 @@
       <c r="AD69" s="42"/>
       <c r="AE69" s="55"/>
     </row>
-    <row r="70" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="23" t="s">
         <v>62</v>
       </c>
@@ -8857,7 +9123,7 @@
       <c r="AD70" s="42"/>
       <c r="AE70" s="55"/>
     </row>
-    <row r="71" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="23" t="s">
         <v>63</v>
       </c>
@@ -8948,7 +9214,7 @@
       <c r="AD71" s="42"/>
       <c r="AE71" s="55"/>
     </row>
-    <row r="72" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="23" t="s">
         <v>64</v>
       </c>
@@ -9039,7 +9305,7 @@
       <c r="AD72" s="42"/>
       <c r="AE72" s="55"/>
     </row>
-    <row r="73" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="23" t="s">
         <v>65</v>
       </c>
@@ -9130,7 +9396,7 @@
       <c r="AD73" s="42"/>
       <c r="AE73" s="55"/>
     </row>
-    <row r="74" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="23" t="s">
         <v>66</v>
       </c>
@@ -9221,7 +9487,7 @@
       <c r="AD74" s="42"/>
       <c r="AE74" s="55"/>
     </row>
-    <row r="75" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="23" t="s">
         <v>67</v>
       </c>
@@ -9312,7 +9578,7 @@
       <c r="AD75" s="42"/>
       <c r="AE75" s="55"/>
     </row>
-    <row r="76" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="23" t="s">
         <v>68</v>
       </c>
@@ -9403,7 +9669,7 @@
       <c r="AD76" s="42"/>
       <c r="AE76" s="55"/>
     </row>
-    <row r="77" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="23" t="s">
         <v>69</v>
       </c>
@@ -9494,7 +9760,7 @@
       <c r="AD77" s="42"/>
       <c r="AE77" s="55"/>
     </row>
-    <row r="78" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="23" t="s">
         <v>70</v>
       </c>
@@ -9585,7 +9851,7 @@
       <c r="AD78" s="42"/>
       <c r="AE78" s="55"/>
     </row>
-    <row r="79" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="23" t="s">
         <v>71</v>
       </c>
@@ -9676,7 +9942,7 @@
       <c r="AD79" s="42"/>
       <c r="AE79" s="55"/>
     </row>
-    <row r="80" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="23" t="s">
         <v>72</v>
       </c>
@@ -9767,7 +10033,7 @@
       <c r="AD80" s="42"/>
       <c r="AE80" s="55"/>
     </row>
-    <row r="81" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="23" t="s">
         <v>73</v>
       </c>
@@ -9858,7 +10124,7 @@
       <c r="AD81" s="42"/>
       <c r="AE81" s="55"/>
     </row>
-    <row r="82" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="23" t="s">
         <v>74</v>
       </c>
@@ -9949,7 +10215,7 @@
       <c r="AD82" s="42"/>
       <c r="AE82" s="55"/>
     </row>
-    <row r="83" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="23" t="s">
         <v>75</v>
       </c>
@@ -10040,7 +10306,7 @@
       <c r="AD83" s="42"/>
       <c r="AE83" s="55"/>
     </row>
-    <row r="84" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="23" t="s">
         <v>76</v>
       </c>
@@ -10131,7 +10397,7 @@
       <c r="AD84" s="42"/>
       <c r="AE84" s="55"/>
     </row>
-    <row r="85" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="23" t="s">
         <v>77</v>
       </c>
@@ -10222,7 +10488,7 @@
       <c r="AD85" s="42"/>
       <c r="AE85" s="55"/>
     </row>
-    <row r="86" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="23" t="s">
         <v>78</v>
       </c>
@@ -10313,7 +10579,7 @@
       <c r="AD86" s="42"/>
       <c r="AE86" s="55"/>
     </row>
-    <row r="87" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="23" t="s">
         <v>79</v>
       </c>
@@ -10404,7 +10670,7 @@
       <c r="AD87" s="42"/>
       <c r="AE87" s="55"/>
     </row>
-    <row r="88" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="23" t="s">
         <v>80</v>
       </c>
@@ -10495,7 +10761,7 @@
       <c r="AD88" s="42"/>
       <c r="AE88" s="55"/>
     </row>
-    <row r="89" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="23" t="s">
         <v>81</v>
       </c>
@@ -10586,7 +10852,7 @@
       <c r="AD89" s="42"/>
       <c r="AE89" s="55"/>
     </row>
-    <row r="90" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="23" t="s">
         <v>82</v>
       </c>
@@ -10677,7 +10943,7 @@
       <c r="AD90" s="42"/>
       <c r="AE90" s="55"/>
     </row>
-    <row r="91" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="23" t="s">
         <v>83</v>
       </c>
@@ -10768,7 +11034,7 @@
       <c r="AD91" s="42"/>
       <c r="AE91" s="55"/>
     </row>
-    <row r="92" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="23" t="s">
         <v>84</v>
       </c>
@@ -10859,7 +11125,7 @@
       <c r="AD92" s="42"/>
       <c r="AE92" s="55"/>
     </row>
-    <row r="93" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="23" t="s">
         <v>85</v>
       </c>
@@ -10950,7 +11216,7 @@
       <c r="AD93" s="42"/>
       <c r="AE93" s="55"/>
     </row>
-    <row r="94" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="23" t="s">
         <v>86</v>
       </c>
@@ -11041,7 +11307,7 @@
       <c r="AD94" s="42"/>
       <c r="AE94" s="55"/>
     </row>
-    <row r="95" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="23" t="s">
         <v>87</v>
       </c>
@@ -11132,7 +11398,7 @@
       <c r="AD95" s="42"/>
       <c r="AE95" s="55"/>
     </row>
-    <row r="96" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="23" t="s">
         <v>88</v>
       </c>
@@ -11223,7 +11489,7 @@
       <c r="AD96" s="42"/>
       <c r="AE96" s="55"/>
     </row>
-    <row r="97" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="23" t="s">
         <v>89</v>
       </c>
@@ -11314,7 +11580,7 @@
       <c r="AD97" s="42"/>
       <c r="AE97" s="55"/>
     </row>
-    <row r="98" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="23" t="s">
         <v>90</v>
       </c>
@@ -11405,7 +11671,7 @@
       <c r="AD98" s="42"/>
       <c r="AE98" s="55"/>
     </row>
-    <row r="99" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="23" t="s">
         <v>91</v>
       </c>
@@ -11496,7 +11762,7 @@
       <c r="AD99" s="42"/>
       <c r="AE99" s="55"/>
     </row>
-    <row r="100" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="23" t="s">
         <v>92</v>
       </c>
@@ -11587,7 +11853,7 @@
       <c r="AD100" s="42"/>
       <c r="AE100" s="55"/>
     </row>
-    <row r="101" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="13"/>
       <c r="B101" s="8"/>
       <c r="C101" s="8"/>
@@ -11620,7 +11886,7 @@
       <c r="AD101" s="42"/>
       <c r="AE101" s="55"/>
     </row>
-    <row r="102" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="13"/>
       <c r="B102" s="8"/>
       <c r="C102" s="8"/>
@@ -11653,7 +11919,7 @@
       <c r="AD102" s="42"/>
       <c r="AE102" s="55"/>
     </row>
-    <row r="103" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="15" t="s">
         <v>95</v>
       </c>
@@ -11690,58 +11956,58 @@
       <c r="AD103" s="42"/>
       <c r="AE103" s="55"/>
     </row>
-    <row r="104" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A104" s="140" t="s">
+    <row r="104" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="141" t="s">
         <v>25</v>
       </c>
-      <c r="B104" s="140"/>
-      <c r="C104" s="140"/>
-      <c r="D104" s="140"/>
-      <c r="E104" s="140"/>
-      <c r="F104" s="140"/>
-      <c r="G104" s="140"/>
-      <c r="H104" s="140"/>
-      <c r="I104" s="140"/>
-      <c r="J104" s="140"/>
-      <c r="K104" s="140"/>
+      <c r="B104" s="141"/>
+      <c r="C104" s="141"/>
+      <c r="D104" s="141"/>
+      <c r="E104" s="141"/>
+      <c r="F104" s="141"/>
+      <c r="G104" s="141"/>
+      <c r="H104" s="141"/>
+      <c r="I104" s="141"/>
+      <c r="J104" s="141"/>
+      <c r="K104" s="141"/>
       <c r="L104" s="8"/>
       <c r="M104" s="8"/>
       <c r="N104" s="8"/>
       <c r="O104" s="14"/>
       <c r="P104" s="54"/>
       <c r="Q104" s="42"/>
-      <c r="R104" s="144" t="s">
+      <c r="R104" s="145" t="s">
         <v>25</v>
       </c>
-      <c r="S104" s="144"/>
-      <c r="T104" s="144"/>
-      <c r="U104" s="144"/>
-      <c r="V104" s="144"/>
-      <c r="W104" s="144"/>
-      <c r="X104" s="144"/>
-      <c r="Y104" s="144"/>
-      <c r="Z104" s="144"/>
-      <c r="AA104" s="144"/>
-      <c r="AB104" s="144"/>
+      <c r="S104" s="145"/>
+      <c r="T104" s="145"/>
+      <c r="U104" s="145"/>
+      <c r="V104" s="145"/>
+      <c r="W104" s="145"/>
+      <c r="X104" s="145"/>
+      <c r="Y104" s="145"/>
+      <c r="Z104" s="145"/>
+      <c r="AA104" s="145"/>
+      <c r="AB104" s="145"/>
       <c r="AD104" s="42"/>
       <c r="AE104" s="55"/>
     </row>
-    <row r="105" spans="1:31" s="36" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:31" s="36" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="102"/>
-      <c r="B105" s="154" t="s">
+      <c r="B105" s="156" t="s">
         <v>55</v>
       </c>
-      <c r="C105" s="155"/>
-      <c r="D105" s="155"/>
-      <c r="E105" s="155"/>
-      <c r="F105" s="155"/>
-      <c r="G105" s="155"/>
-      <c r="H105" s="156"/>
-      <c r="I105" s="151" t="s">
+      <c r="C105" s="157"/>
+      <c r="D105" s="157"/>
+      <c r="E105" s="157"/>
+      <c r="F105" s="157"/>
+      <c r="G105" s="157"/>
+      <c r="H105" s="158"/>
+      <c r="I105" s="153" t="s">
         <v>1</v>
       </c>
-      <c r="J105" s="152"/>
-      <c r="K105" s="153"/>
+      <c r="J105" s="154"/>
+      <c r="K105" s="155"/>
       <c r="L105" s="8"/>
       <c r="M105" s="8"/>
       <c r="N105" s="8"/>
@@ -11749,15 +12015,15 @@
       <c r="P105" s="54"/>
       <c r="Q105" s="42"/>
       <c r="R105" s="45"/>
-      <c r="S105" s="145" t="s">
+      <c r="S105" s="146" t="s">
         <v>55</v>
       </c>
-      <c r="T105" s="145"/>
-      <c r="U105" s="145"/>
-      <c r="V105" s="145"/>
-      <c r="W105" s="145"/>
-      <c r="X105" s="145"/>
-      <c r="Y105" s="145"/>
+      <c r="T105" s="146"/>
+      <c r="U105" s="146"/>
+      <c r="V105" s="146"/>
+      <c r="W105" s="146"/>
+      <c r="X105" s="146"/>
+      <c r="Y105" s="146"/>
       <c r="Z105" s="103" t="s">
         <v>1</v>
       </c>
@@ -11767,7 +12033,7 @@
       <c r="AD105" s="42"/>
       <c r="AE105" s="55"/>
     </row>
-    <row r="106" spans="1:31" s="36" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:31" s="36" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>56</v>
       </c>
@@ -11848,7 +12114,7 @@
       <c r="AD106" s="42"/>
       <c r="AE106" s="55"/>
     </row>
-    <row r="107" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="23" t="s">
         <v>57</v>
       </c>
@@ -11939,7 +12205,7 @@
       <c r="AD107" s="42"/>
       <c r="AE107" s="55"/>
     </row>
-    <row r="108" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="23" t="s">
         <v>58</v>
       </c>
@@ -12030,7 +12296,7 @@
       <c r="AD108" s="42"/>
       <c r="AE108" s="55"/>
     </row>
-    <row r="109" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="23" t="s">
         <v>59</v>
       </c>
@@ -12121,7 +12387,7 @@
       <c r="AD109" s="42"/>
       <c r="AE109" s="55"/>
     </row>
-    <row r="110" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="23" t="s">
         <v>60</v>
       </c>
@@ -12212,7 +12478,7 @@
       <c r="AD110" s="42"/>
       <c r="AE110" s="55"/>
     </row>
-    <row r="111" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="23" t="s">
         <v>61</v>
       </c>
@@ -12303,7 +12569,7 @@
       <c r="AD111" s="42"/>
       <c r="AE111" s="55"/>
     </row>
-    <row r="112" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="23" t="s">
         <v>62</v>
       </c>
@@ -12391,7 +12657,7 @@
       <c r="AD112" s="42"/>
       <c r="AE112" s="55"/>
     </row>
-    <row r="113" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="23" t="s">
         <v>63</v>
       </c>
@@ -12482,7 +12748,7 @@
       <c r="AD113" s="42"/>
       <c r="AE113" s="55"/>
     </row>
-    <row r="114" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="23" t="s">
         <v>64</v>
       </c>
@@ -12573,7 +12839,7 @@
       <c r="AD114" s="42"/>
       <c r="AE114" s="55"/>
     </row>
-    <row r="115" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="23" t="s">
         <v>65</v>
       </c>
@@ -12664,7 +12930,7 @@
       <c r="AD115" s="42"/>
       <c r="AE115" s="55"/>
     </row>
-    <row r="116" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="23" t="s">
         <v>66</v>
       </c>
@@ -12755,7 +13021,7 @@
       <c r="AD116" s="42"/>
       <c r="AE116" s="55"/>
     </row>
-    <row r="117" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="23" t="s">
         <v>67</v>
       </c>
@@ -12846,7 +13112,7 @@
       <c r="AD117" s="42"/>
       <c r="AE117" s="55"/>
     </row>
-    <row r="118" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="23" t="s">
         <v>68</v>
       </c>
@@ -12937,7 +13203,7 @@
       <c r="AD118" s="42"/>
       <c r="AE118" s="55"/>
     </row>
-    <row r="119" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="23" t="s">
         <v>69</v>
       </c>
@@ -13028,7 +13294,7 @@
       <c r="AD119" s="42"/>
       <c r="AE119" s="55"/>
     </row>
-    <row r="120" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="23" t="s">
         <v>70</v>
       </c>
@@ -13119,7 +13385,7 @@
       <c r="AD120" s="42"/>
       <c r="AE120" s="55"/>
     </row>
-    <row r="121" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="23" t="s">
         <v>71</v>
       </c>
@@ -13210,7 +13476,7 @@
       <c r="AD121" s="42"/>
       <c r="AE121" s="55"/>
     </row>
-    <row r="122" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="23" t="s">
         <v>72</v>
       </c>
@@ -13301,7 +13567,7 @@
       <c r="AD122" s="42"/>
       <c r="AE122" s="55"/>
     </row>
-    <row r="123" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="23" t="s">
         <v>73</v>
       </c>
@@ -13392,7 +13658,7 @@
       <c r="AD123" s="42"/>
       <c r="AE123" s="55"/>
     </row>
-    <row r="124" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="23" t="s">
         <v>74</v>
       </c>
@@ -13483,7 +13749,7 @@
       <c r="AD124" s="42"/>
       <c r="AE124" s="55"/>
     </row>
-    <row r="125" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="23" t="s">
         <v>75</v>
       </c>
@@ -13574,7 +13840,7 @@
       <c r="AD125" s="42"/>
       <c r="AE125" s="55"/>
     </row>
-    <row r="126" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="23" t="s">
         <v>76</v>
       </c>
@@ -13665,7 +13931,7 @@
       <c r="AD126" s="42"/>
       <c r="AE126" s="55"/>
     </row>
-    <row r="127" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="23" t="s">
         <v>77</v>
       </c>
@@ -13756,7 +14022,7 @@
       <c r="AD127" s="42"/>
       <c r="AE127" s="55"/>
     </row>
-    <row r="128" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="23" t="s">
         <v>78</v>
       </c>
@@ -13847,7 +14113,7 @@
       <c r="AD128" s="42"/>
       <c r="AE128" s="55"/>
     </row>
-    <row r="129" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="23" t="s">
         <v>79</v>
       </c>
@@ -13938,7 +14204,7 @@
       <c r="AD129" s="42"/>
       <c r="AE129" s="55"/>
     </row>
-    <row r="130" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="23" t="s">
         <v>80</v>
       </c>
@@ -14028,7 +14294,7 @@
       <c r="AD130" s="42"/>
       <c r="AE130" s="55"/>
     </row>
-    <row r="131" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="23" t="s">
         <v>81</v>
       </c>
@@ -14119,7 +14385,7 @@
       <c r="AD131" s="42"/>
       <c r="AE131" s="55"/>
     </row>
-    <row r="132" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="23" t="s">
         <v>82</v>
       </c>
@@ -14210,7 +14476,7 @@
       <c r="AD132" s="42"/>
       <c r="AE132" s="55"/>
     </row>
-    <row r="133" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="23" t="s">
         <v>83</v>
       </c>
@@ -14301,7 +14567,7 @@
       <c r="AD133" s="42"/>
       <c r="AE133" s="55"/>
     </row>
-    <row r="134" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="23" t="s">
         <v>84</v>
       </c>
@@ -14392,7 +14658,7 @@
       <c r="AD134" s="42"/>
       <c r="AE134" s="55"/>
     </row>
-    <row r="135" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="23" t="s">
         <v>85</v>
       </c>
@@ -14483,7 +14749,7 @@
       <c r="AD135" s="42"/>
       <c r="AE135" s="55"/>
     </row>
-    <row r="136" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="23" t="s">
         <v>86</v>
       </c>
@@ -14574,7 +14840,7 @@
       <c r="AD136" s="42"/>
       <c r="AE136" s="55"/>
     </row>
-    <row r="137" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="23" t="s">
         <v>87</v>
       </c>
@@ -14665,7 +14931,7 @@
       <c r="AD137" s="42"/>
       <c r="AE137" s="55"/>
     </row>
-    <row r="138" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="23" t="s">
         <v>88</v>
       </c>
@@ -14756,7 +15022,7 @@
       <c r="AD138" s="42"/>
       <c r="AE138" s="55"/>
     </row>
-    <row r="139" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="23" t="s">
         <v>89</v>
       </c>
@@ -14847,7 +15113,7 @@
       <c r="AD139" s="42"/>
       <c r="AE139" s="55"/>
     </row>
-    <row r="140" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A140" s="23" t="s">
         <v>90</v>
       </c>
@@ -14938,7 +15204,7 @@
       <c r="AD140" s="42"/>
       <c r="AE140" s="55"/>
     </row>
-    <row r="141" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A141" s="23" t="s">
         <v>91</v>
       </c>
@@ -15029,7 +15295,7 @@
       <c r="AD141" s="42"/>
       <c r="AE141" s="55"/>
     </row>
-    <row r="142" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="23" t="s">
         <v>92</v>
       </c>
@@ -15120,7 +15386,7 @@
       <c r="AD142" s="42"/>
       <c r="AE142" s="55"/>
     </row>
-    <row r="143" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A143" s="13"/>
       <c r="B143" s="8"/>
       <c r="C143" s="8"/>
@@ -15153,7 +15419,7 @@
       <c r="AD143" s="42"/>
       <c r="AE143" s="55"/>
     </row>
-    <row r="144" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="13"/>
       <c r="B144" s="8"/>
       <c r="C144" s="8"/>
@@ -15186,7 +15452,7 @@
       <c r="AD144" s="42"/>
       <c r="AE144" s="55"/>
     </row>
-    <row r="145" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="13"/>
       <c r="B145" s="8"/>
       <c r="C145" s="8"/>
@@ -15219,7 +15485,7 @@
       <c r="AD145" s="42"/>
       <c r="AE145" s="55"/>
     </row>
-    <row r="146" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A146" s="13"/>
       <c r="B146" s="8"/>
       <c r="C146" s="8"/>
@@ -15252,7 +15518,7 @@
       <c r="AD146" s="42"/>
       <c r="AE146" s="55"/>
     </row>
-    <row r="147" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="13"/>
       <c r="B147" s="8"/>
       <c r="C147" s="8"/>
@@ -15285,7 +15551,7 @@
       <c r="AD147" s="42"/>
       <c r="AE147" s="55"/>
     </row>
-    <row r="148" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A148" s="13"/>
       <c r="B148" s="8"/>
       <c r="C148" s="8"/>
@@ -15318,7 +15584,7 @@
       <c r="AD148" s="42"/>
       <c r="AE148" s="55"/>
     </row>
-    <row r="149" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A149" s="13"/>
       <c r="B149" s="8"/>
       <c r="C149" s="8"/>
@@ -15351,7 +15617,7 @@
       <c r="AD149" s="42"/>
       <c r="AE149" s="55"/>
     </row>
-    <row r="150" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A150" s="13"/>
       <c r="B150" s="8"/>
       <c r="C150" s="8"/>
@@ -15384,7 +15650,7 @@
       <c r="AD150" s="42"/>
       <c r="AE150" s="55"/>
     </row>
-    <row r="151" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A151" s="13"/>
       <c r="B151" s="8"/>
       <c r="C151" s="8"/>
@@ -15417,7 +15683,7 @@
       <c r="AD151" s="42"/>
       <c r="AE151" s="55"/>
     </row>
-    <row r="152" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:31" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A152" s="13"/>
       <c r="B152" s="8"/>
       <c r="C152" s="8"/>
@@ -15450,204 +15716,199 @@
       <c r="AD152" s="42"/>
       <c r="AE152" s="55"/>
     </row>
-    <row r="158" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="B158" s="146"/>
-      <c r="C158" s="146"/>
-      <c r="D158" s="146"/>
-    </row>
-    <row r="159" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="B158" s="148"/>
+      <c r="C158" s="148"/>
+      <c r="D158" s="148"/>
+    </row>
+    <row r="159" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A159" s="15"/>
       <c r="B159" s="65"/>
       <c r="C159" s="65"/>
       <c r="D159" s="65"/>
     </row>
-    <row r="160" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A160" s="66"/>
       <c r="D160" s="60"/>
       <c r="F160" s="62"/>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" s="66"/>
       <c r="D161" s="60"/>
       <c r="F161" s="62"/>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A162" s="66"/>
       <c r="D162" s="60"/>
       <c r="F162" s="62"/>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" s="66"/>
       <c r="D163" s="60"/>
       <c r="F163" s="62"/>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A164" s="66"/>
       <c r="D164" s="60"/>
       <c r="F164" s="62"/>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A165" s="66"/>
       <c r="D165" s="60"/>
       <c r="F165" s="62"/>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A166" s="66"/>
       <c r="D166" s="60"/>
       <c r="F166" s="62"/>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A167" s="66"/>
       <c r="D167" s="60"/>
       <c r="F167" s="62"/>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A168" s="66"/>
       <c r="D168" s="60"/>
       <c r="F168" s="62"/>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A169" s="66"/>
       <c r="D169" s="60"/>
       <c r="F169" s="62"/>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A170" s="66"/>
       <c r="D170" s="60"/>
       <c r="F170" s="62"/>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A171" s="66"/>
       <c r="D171" s="60"/>
       <c r="F171" s="62"/>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A172" s="66"/>
       <c r="D172" s="60"/>
       <c r="F172" s="62"/>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A173" s="66"/>
       <c r="D173" s="60"/>
       <c r="F173" s="62"/>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A174" s="66"/>
       <c r="D174" s="60"/>
       <c r="F174" s="62"/>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A175" s="66"/>
       <c r="D175" s="60"/>
       <c r="F175" s="62"/>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A176" s="66"/>
       <c r="D176" s="60"/>
       <c r="F176" s="62"/>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A177" s="66"/>
       <c r="D177" s="60"/>
       <c r="F177" s="62"/>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A178" s="66"/>
       <c r="D178" s="60"/>
       <c r="F178" s="62"/>
     </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A179" s="66"/>
       <c r="D179" s="60"/>
       <c r="F179" s="62"/>
     </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A180" s="66"/>
       <c r="D180" s="60"/>
       <c r="F180" s="62"/>
     </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A181" s="66"/>
       <c r="D181" s="60"/>
       <c r="F181" s="62"/>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A182" s="66"/>
       <c r="D182" s="60"/>
       <c r="F182" s="62"/>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A183" s="66"/>
       <c r="D183" s="60"/>
       <c r="F183" s="62"/>
     </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A184" s="66"/>
       <c r="D184" s="60"/>
       <c r="F184" s="62"/>
     </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A185" s="66"/>
       <c r="D185" s="60"/>
       <c r="F185" s="62"/>
     </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A186" s="66"/>
       <c r="D186" s="60"/>
       <c r="F186" s="62"/>
     </row>
-    <row r="187" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A187" s="66"/>
       <c r="D187" s="60"/>
       <c r="F187" s="62"/>
     </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A188" s="66"/>
       <c r="D188" s="60"/>
       <c r="F188" s="62"/>
     </row>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A189" s="66"/>
       <c r="D189" s="60"/>
       <c r="F189" s="62"/>
     </row>
-    <row r="190" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A190" s="66"/>
       <c r="D190" s="60"/>
       <c r="F190" s="62"/>
     </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A191" s="66"/>
       <c r="D191" s="60"/>
       <c r="F191" s="62"/>
     </row>
-    <row r="192" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A192" s="66"/>
       <c r="D192" s="60"/>
       <c r="F192" s="62"/>
     </row>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A193" s="66"/>
       <c r="D193" s="60"/>
       <c r="F193" s="62"/>
     </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A194" s="66"/>
       <c r="D194" s="60"/>
       <c r="F194" s="62"/>
     </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A195" s="66"/>
       <c r="D195" s="60"/>
       <c r="F195" s="62"/>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="P1:AE1"/>
-    <mergeCell ref="A62:K62"/>
-    <mergeCell ref="R62:AB62"/>
     <mergeCell ref="R104:AB104"/>
     <mergeCell ref="S105:Y105"/>
     <mergeCell ref="B158:D158"/>
@@ -15657,64 +15918,69 @@
     <mergeCell ref="B105:H105"/>
     <mergeCell ref="A104:K104"/>
     <mergeCell ref="S63:Y63"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="P1:AE1"/>
+    <mergeCell ref="A62:K62"/>
+    <mergeCell ref="R62:AB62"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AD18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.26953125" style="13" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" style="8" customWidth="1"/>
-    <col min="3" max="3" width="14.26953125" style="8" customWidth="1"/>
-    <col min="4" max="13" width="8.7265625" style="8"/>
-    <col min="14" max="14" width="8.7265625" style="14"/>
-    <col min="15" max="15" width="8.7265625" style="36"/>
+    <col min="1" max="1" width="12.28515625" style="13" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" style="8" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" style="8" customWidth="1"/>
+    <col min="4" max="13" width="8.7109375" style="8"/>
+    <col min="14" max="14" width="8.7109375" style="14"/>
+    <col min="15" max="15" width="8.7109375" style="36"/>
     <col min="16" max="16" width="15" style="36" customWidth="1"/>
-    <col min="17" max="30" width="8.7265625" style="36"/>
+    <col min="17" max="30" width="8.7109375" style="36"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="29" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="137" t="s">
+    <row r="1" spans="1:30" ht="29.25" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="138" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="138"/>
-      <c r="C1" s="138"/>
-      <c r="D1" s="138"/>
-      <c r="E1" s="138"/>
-      <c r="F1" s="138"/>
-      <c r="G1" s="138"/>
-      <c r="H1" s="138"/>
-      <c r="I1" s="138"/>
-      <c r="J1" s="138"/>
-      <c r="K1" s="138"/>
-      <c r="L1" s="138"/>
-      <c r="M1" s="138"/>
-      <c r="N1" s="141"/>
-      <c r="O1" s="135" t="s">
+      <c r="B1" s="139"/>
+      <c r="C1" s="139"/>
+      <c r="D1" s="139"/>
+      <c r="E1" s="139"/>
+      <c r="F1" s="139"/>
+      <c r="G1" s="139"/>
+      <c r="H1" s="139"/>
+      <c r="I1" s="139"/>
+      <c r="J1" s="139"/>
+      <c r="K1" s="139"/>
+      <c r="L1" s="139"/>
+      <c r="M1" s="139"/>
+      <c r="N1" s="142"/>
+      <c r="O1" s="136" t="s">
         <v>50</v>
       </c>
-      <c r="P1" s="136"/>
-      <c r="Q1" s="136"/>
-      <c r="R1" s="136"/>
-      <c r="S1" s="136"/>
-      <c r="T1" s="136"/>
-      <c r="U1" s="136"/>
-      <c r="V1" s="136"/>
-      <c r="W1" s="136"/>
-      <c r="X1" s="136"/>
-      <c r="Y1" s="136"/>
-      <c r="Z1" s="136"/>
-      <c r="AA1" s="136"/>
-      <c r="AB1" s="136"/>
-      <c r="AC1" s="136"/>
-      <c r="AD1" s="139"/>
-    </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.35">
+      <c r="P1" s="137"/>
+      <c r="Q1" s="137"/>
+      <c r="R1" s="137"/>
+      <c r="S1" s="137"/>
+      <c r="T1" s="137"/>
+      <c r="U1" s="137"/>
+      <c r="V1" s="137"/>
+      <c r="W1" s="137"/>
+      <c r="X1" s="137"/>
+      <c r="Y1" s="137"/>
+      <c r="Z1" s="137"/>
+      <c r="AA1" s="137"/>
+      <c r="AB1" s="137"/>
+      <c r="AC1" s="137"/>
+      <c r="AD1" s="140"/>
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
         <v>13</v>
       </c>
@@ -15724,7 +15990,7 @@
       <c r="Q3" s="42"/>
       <c r="R3" s="42"/>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
         <v>31</v>
       </c>
@@ -15738,7 +16004,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
         <v>129</v>
       </c>
@@ -15754,15 +16020,15 @@
         <v>5.6366197183098592</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="15"/>
       <c r="P6" s="47"/>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="15"/>
       <c r="P7" s="47"/>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="16" t="s">
         <v>31</v>
       </c>
@@ -15782,7 +16048,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="95" t="s">
         <v>129</v>
       </c>
@@ -15806,19 +16072,19 @@
         <v>7.4281690140845065</v>
       </c>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="15"/>
       <c r="P10" s="47"/>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="15"/>
       <c r="P11" s="47"/>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="15"/>
       <c r="P12" s="47"/>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
         <v>129</v>
       </c>
@@ -15886,7 +16152,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="16" t="s">
         <v>24</v>
       </c>
@@ -15954,7 +16220,7 @@
         <v>6.3464788732394375</v>
       </c>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="s">
         <v>25</v>
       </c>
@@ -16022,10 +16288,10 @@
         <v>5.1464788732394364</v>
       </c>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
       <c r="P16" s="47"/>
     </row>
-    <row r="17" spans="2:26" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B17" s="63"/>
       <c r="C17" s="63"/>
       <c r="D17" s="63"/>
@@ -16038,7 +16304,7 @@
       <c r="K17" s="63"/>
       <c r="P17" s="47"/>
     </row>
-    <row r="18" spans="2:26" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B18" s="63"/>
       <c r="C18" s="63"/>
       <c r="D18" s="63"/>
@@ -16099,21 +16365,21 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="C4:J9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="22.6328125" customWidth="1"/>
-    <col min="4" max="4" width="13.6328125" customWidth="1"/>
-    <col min="5" max="5" width="14.7265625" customWidth="1"/>
-    <col min="6" max="6" width="11.1796875" customWidth="1"/>
-    <col min="7" max="7" width="10.26953125" customWidth="1"/>
-    <col min="8" max="8" width="10.6328125" customWidth="1"/>
-    <col min="10" max="10" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.5703125" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.140625" customWidth="1"/>
+    <col min="7" max="7" width="10.28515625" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" customWidth="1"/>
+    <col min="10" max="10" width="13.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C4" s="79" t="s">
         <v>31</v>
       </c>
@@ -16133,7 +16399,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="5" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C5" s="80" t="s">
         <v>41</v>
       </c>
@@ -16155,7 +16421,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="6" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C6" s="80" t="s">
         <v>120</v>
       </c>
@@ -16175,7 +16441,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="7" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C7" s="80" t="s">
         <v>108</v>
       </c>
@@ -16198,7 +16464,7 @@
       </c>
       <c r="J7" s="78"/>
     </row>
-    <row r="8" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C8" s="80" t="s">
         <v>128</v>
       </c>
@@ -16219,7 +16485,7 @@
       </c>
       <c r="J8" s="78"/>
     </row>
-    <row r="9" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C9" s="80" t="s">
         <v>125</v>
       </c>
@@ -16249,65 +16515,65 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AD101"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.26953125" style="13" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" style="8" customWidth="1"/>
-    <col min="3" max="3" width="14.26953125" style="8" customWidth="1"/>
-    <col min="4" max="7" width="8.7265625" style="8"/>
-    <col min="8" max="8" width="14.36328125" style="8" customWidth="1"/>
-    <col min="9" max="9" width="13.453125" style="8" customWidth="1"/>
-    <col min="10" max="13" width="8.7265625" style="8"/>
-    <col min="14" max="14" width="8.7265625" style="14"/>
-    <col min="15" max="15" width="12.26953125" style="54" customWidth="1"/>
-    <col min="16" max="16" width="12.6328125" style="42" customWidth="1"/>
-    <col min="17" max="17" width="10.453125" style="111" customWidth="1"/>
+    <col min="1" max="1" width="12.28515625" style="13" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" style="8" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" style="8" customWidth="1"/>
+    <col min="4" max="7" width="8.7109375" style="8"/>
+    <col min="8" max="8" width="14.42578125" style="8" customWidth="1"/>
+    <col min="9" max="9" width="13.42578125" style="8" customWidth="1"/>
+    <col min="10" max="13" width="8.7109375" style="8"/>
+    <col min="14" max="14" width="8.7109375" style="14"/>
+    <col min="15" max="15" width="12.28515625" style="54" customWidth="1"/>
+    <col min="16" max="16" width="12.5703125" style="42" customWidth="1"/>
+    <col min="17" max="17" width="10.42578125" style="111" customWidth="1"/>
     <col min="18" max="20" width="10" style="111" customWidth="1"/>
-    <col min="21" max="21" width="12.90625" style="111" customWidth="1"/>
-    <col min="22" max="22" width="17.7265625" style="111" customWidth="1"/>
-    <col min="23" max="23" width="17.08984375" style="42" customWidth="1"/>
-    <col min="24" max="29" width="8.7265625" style="42"/>
-    <col min="30" max="30" width="8.7265625" style="55"/>
+    <col min="21" max="21" width="12.85546875" style="111" customWidth="1"/>
+    <col min="22" max="22" width="17.7109375" style="111" customWidth="1"/>
+    <col min="23" max="23" width="17.140625" style="42" customWidth="1"/>
+    <col min="24" max="29" width="8.7109375" style="42"/>
+    <col min="30" max="30" width="8.7109375" style="55"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="29" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="158"/>
-      <c r="B1" s="159"/>
-      <c r="C1" s="159"/>
-      <c r="D1" s="159"/>
-      <c r="E1" s="159"/>
-      <c r="F1" s="159"/>
-      <c r="G1" s="159"/>
-      <c r="H1" s="159"/>
-      <c r="I1" s="159"/>
-      <c r="J1" s="159"/>
-      <c r="K1" s="159"/>
-      <c r="L1" s="159"/>
-      <c r="M1" s="159"/>
-      <c r="N1" s="160"/>
-      <c r="O1" s="135" t="s">
+    <row r="1" spans="1:30" ht="29.25" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="159"/>
+      <c r="B1" s="160"/>
+      <c r="C1" s="160"/>
+      <c r="D1" s="160"/>
+      <c r="E1" s="160"/>
+      <c r="F1" s="160"/>
+      <c r="G1" s="160"/>
+      <c r="H1" s="160"/>
+      <c r="I1" s="160"/>
+      <c r="J1" s="160"/>
+      <c r="K1" s="160"/>
+      <c r="L1" s="160"/>
+      <c r="M1" s="160"/>
+      <c r="N1" s="161"/>
+      <c r="O1" s="136" t="s">
         <v>50</v>
       </c>
-      <c r="P1" s="136"/>
-      <c r="Q1" s="136"/>
-      <c r="R1" s="136"/>
-      <c r="S1" s="136"/>
-      <c r="T1" s="136"/>
-      <c r="U1" s="136"/>
-      <c r="V1" s="136"/>
-      <c r="W1" s="136"/>
-      <c r="X1" s="136"/>
-      <c r="Y1" s="136"/>
-      <c r="Z1" s="136"/>
-      <c r="AA1" s="136"/>
-      <c r="AB1" s="136"/>
-      <c r="AC1" s="136"/>
-      <c r="AD1" s="139"/>
-    </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.35">
+      <c r="P1" s="137"/>
+      <c r="Q1" s="137"/>
+      <c r="R1" s="137"/>
+      <c r="S1" s="137"/>
+      <c r="T1" s="137"/>
+      <c r="U1" s="137"/>
+      <c r="V1" s="137"/>
+      <c r="W1" s="137"/>
+      <c r="X1" s="137"/>
+      <c r="Y1" s="137"/>
+      <c r="Z1" s="137"/>
+      <c r="AA1" s="137"/>
+      <c r="AB1" s="137"/>
+      <c r="AC1" s="137"/>
+      <c r="AD1" s="140"/>
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B3" s="96" t="s">
         <v>13</v>
       </c>
@@ -16322,7 +16588,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:30" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:30" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="31" t="s">
         <v>142</v>
       </c>
@@ -16371,7 +16637,7 @@
       <c r="AA4" s="108"/>
       <c r="AB4" s="108"/>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B5" s="31" t="s">
         <v>1</v>
       </c>
@@ -16427,7 +16693,7 @@
       <c r="AA5" s="118"/>
       <c r="AB5" s="118"/>
     </row>
-    <row r="6" spans="1:30" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:30" ht="30" x14ac:dyDescent="0.25">
       <c r="B6" s="31" t="s">
         <v>6</v>
       </c>
@@ -16482,7 +16748,7 @@
       <c r="Z6" s="108"/>
       <c r="AA6" s="108"/>
     </row>
-    <row r="7" spans="1:30" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:30" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="15"/>
       <c r="B7" s="31" t="s">
         <v>150</v>
@@ -16512,13 +16778,13 @@
       <c r="P7" s="52" t="s">
         <v>150</v>
       </c>
-      <c r="Q7" s="161">
+      <c r="Q7" s="132">
         <v>111.205265</v>
       </c>
-      <c r="R7" s="161">
+      <c r="R7" s="132">
         <v>35.099961</v>
       </c>
-      <c r="S7" s="161">
+      <c r="S7" s="132">
         <v>4910.5489479999997</v>
       </c>
       <c r="T7" s="114">
@@ -16538,7 +16804,7 @@
       <c r="Z7" s="118"/>
       <c r="AA7" s="118"/>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="15"/>
       <c r="O8" s="37"/>
       <c r="X8" s="108"/>
@@ -16546,7 +16812,7 @@
       <c r="Z8" s="118"/>
       <c r="AA8" s="118"/>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="15"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -16558,7 +16824,7 @@
       <c r="Z9" s="118"/>
       <c r="AA9" s="118"/>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="107"/>
       <c r="B10" s="127" t="s">
         <v>18</v>
@@ -16575,7 +16841,7 @@
       </c>
       <c r="Q10" s="110"/>
     </row>
-    <row r="11" spans="1:30" ht="47" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:30" ht="47.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="15"/>
       <c r="B11" s="2" t="s">
         <v>27</v>
@@ -16627,7 +16893,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="15"/>
       <c r="B12" s="2" t="s">
         <v>14</v>
@@ -16685,7 +16951,7 @@
         <v>3.3313080260603999E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:30" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:30" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="15"/>
       <c r="B13" s="2" t="s">
         <v>14</v>
@@ -16747,7 +17013,7 @@
       <c r="AB13" s="36"/>
       <c r="AC13" s="36"/>
     </row>
-    <row r="14" spans="1:30" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:30" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="15"/>
       <c r="B14" s="2" t="s">
         <v>14</v>
@@ -16809,7 +17075,7 @@
       <c r="AB14" s="36"/>
       <c r="AC14" s="36"/>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="15"/>
       <c r="B15" s="2" t="s">
         <v>15</v>
@@ -16874,7 +17140,7 @@
       <c r="AB15" s="36"/>
       <c r="AC15" s="36"/>
     </row>
-    <row r="16" spans="1:30" ht="29" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:30" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="15"/>
       <c r="B16" s="2" t="s">
         <v>15</v>
@@ -16939,7 +17205,7 @@
       <c r="AB16" s="36"/>
       <c r="AC16" s="36"/>
     </row>
-    <row r="17" spans="1:25" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:25" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="15"/>
       <c r="B17" s="2" t="s">
         <v>15</v>
@@ -17000,7 +17266,7 @@
       </c>
       <c r="X17" s="64"/>
     </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A18" s="15"/>
       <c r="B18" s="63"/>
       <c r="C18" s="63"/>
@@ -17020,13 +17286,13 @@
       <c r="W18" s="64"/>
       <c r="X18" s="64"/>
     </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
       <c r="J19" s="4"/>
       <c r="K19" s="4"/>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
     </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B20" s="129" t="s">
         <v>146</v>
       </c>
@@ -17054,7 +17320,7 @@
       <c r="X20" s="64"/>
       <c r="Y20" s="64"/>
     </row>
-    <row r="21" spans="1:25" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:25" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="21" t="s">
         <v>48</v>
       </c>
@@ -17106,7 +17372,7 @@
       <c r="X21" s="64"/>
       <c r="Y21" s="64"/>
     </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B22" s="21">
         <v>1</v>
       </c>
@@ -17156,7 +17422,7 @@
         <v>5.7242353618298235E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B23" s="21">
         <v>2</v>
       </c>
@@ -17206,7 +17472,7 @@
         <v>4.9988589140679676E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B24" s="21">
         <v>3</v>
       </c>
@@ -17256,7 +17522,7 @@
         <v>4.6487026288785961E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B25" s="21">
         <v>4</v>
       </c>
@@ -17306,7 +17572,7 @@
         <v>4.4055886058597102E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B26" s="21">
         <v>5</v>
       </c>
@@ -17356,7 +17622,7 @@
         <v>4.1129764331873049E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B27" s="21">
         <v>6</v>
       </c>
@@ -17406,7 +17672,7 @@
         <v>3.8668739037762259E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B28" s="21">
         <v>7</v>
       </c>
@@ -17456,7 +17722,7 @@
         <v>3.6334422789279411E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B29" s="21">
         <v>8</v>
       </c>
@@ -17506,7 +17772,7 @@
         <v>3.3612602818388231E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B30" s="21">
         <v>9</v>
       </c>
@@ -17556,7 +17822,7 @@
         <v>3.0357443519680002E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B31" s="21">
         <v>10</v>
       </c>
@@ -17606,7 +17872,7 @@
         <v>2.3847316141751403E-2</v>
       </c>
     </row>
-    <row r="34" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B34" s="129" t="s">
         <v>147</v>
       </c>
@@ -17620,7 +17886,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="35" spans="2:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:22" ht="75" x14ac:dyDescent="0.25">
       <c r="B35" s="21" t="s">
         <v>48</v>
       </c>
@@ -17664,7 +17930,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="36" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B36" s="21">
         <v>1</v>
       </c>
@@ -17714,7 +17980,7 @@
         <v>4.339861492504693E-2</v>
       </c>
     </row>
-    <row r="37" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B37" s="21">
         <v>2</v>
       </c>
@@ -17764,7 +18030,7 @@
         <v>3.8358034343012805E-2</v>
       </c>
     </row>
-    <row r="38" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B38" s="21">
         <v>3</v>
       </c>
@@ -17814,7 +18080,7 @@
         <v>3.5200779596637477E-2</v>
       </c>
     </row>
-    <row r="39" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B39" s="21">
         <v>4</v>
       </c>
@@ -17864,7 +18130,7 @@
         <v>3.3756258692500582E-2</v>
       </c>
     </row>
-    <row r="40" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B40" s="21">
         <v>5</v>
       </c>
@@ -17914,7 +18180,7 @@
         <v>3.1115350510339534E-2</v>
       </c>
     </row>
-    <row r="41" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B41" s="21">
         <v>6</v>
       </c>
@@ -17964,7 +18230,7 @@
         <v>2.9736482486268499E-2</v>
       </c>
     </row>
-    <row r="42" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B42" s="21">
         <v>7</v>
       </c>
@@ -18014,7 +18280,7 @@
         <v>2.8706754096232103E-2</v>
       </c>
     </row>
-    <row r="43" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B43" s="21">
         <v>8</v>
       </c>
@@ -18064,7 +18330,7 @@
         <v>2.6822213760033416E-2</v>
       </c>
     </row>
-    <row r="44" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B44" s="21">
         <v>9</v>
       </c>
@@ -18114,7 +18380,7 @@
         <v>2.4561578875472542E-2</v>
       </c>
     </row>
-    <row r="45" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B45" s="21">
         <v>10</v>
       </c>
@@ -18164,10 +18430,10 @@
         <v>1.8971720257888285E-2</v>
       </c>
     </row>
-    <row r="47" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:22" x14ac:dyDescent="0.25">
       <c r="P47" s="116"/>
     </row>
-    <row r="48" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B48" s="129" t="s">
         <v>151</v>
       </c>
@@ -18181,7 +18447,7 @@
       <c r="U48" s="42"/>
       <c r="V48" s="42"/>
     </row>
-    <row r="49" spans="2:22" ht="58" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:22" ht="75" x14ac:dyDescent="0.25">
       <c r="B49" s="21" t="s">
         <v>48</v>
       </c>
@@ -18225,7 +18491,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="50" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B50" s="21">
         <v>1</v>
       </c>
@@ -18275,7 +18541,7 @@
         <v>4.6111231162943217E-2</v>
       </c>
     </row>
-    <row r="51" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B51" s="21">
         <v>2</v>
       </c>
@@ -18325,7 +18591,7 @@
         <v>4.1717204364823221E-2</v>
       </c>
     </row>
-    <row r="52" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B52" s="21">
         <v>3</v>
       </c>
@@ -18375,7 +18641,7 @@
         <v>3.9154003953695289E-2</v>
       </c>
     </row>
-    <row r="53" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B53" s="21">
         <v>4</v>
       </c>
@@ -18425,7 +18691,7 @@
         <v>3.7924197640395715E-2</v>
       </c>
     </row>
-    <row r="54" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B54" s="21">
         <v>5</v>
       </c>
@@ -18475,7 +18741,7 @@
         <v>3.5521844764814604E-2</v>
       </c>
     </row>
-    <row r="55" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B55" s="21">
         <v>6</v>
       </c>
@@ -18525,7 +18791,7 @@
         <v>3.4274070804076191E-2</v>
       </c>
     </row>
-    <row r="56" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B56" s="21">
         <v>7</v>
       </c>
@@ -18575,7 +18841,7 @@
         <v>3.3099132864877534E-2</v>
       </c>
     </row>
-    <row r="57" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B57" s="21">
         <v>8</v>
       </c>
@@ -18625,7 +18891,7 @@
         <v>3.11816134057676E-2</v>
       </c>
     </row>
-    <row r="58" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B58" s="21">
         <v>9</v>
       </c>
@@ -18675,7 +18941,7 @@
         <v>2.8740094747443021E-2</v>
       </c>
     </row>
-    <row r="59" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B59" s="21">
         <v>10</v>
       </c>
@@ -18725,13 +18991,13 @@
         <v>2.284074895733508E-2</v>
       </c>
     </row>
-    <row r="60" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:22" x14ac:dyDescent="0.25">
       <c r="P60" s="116"/>
     </row>
-    <row r="61" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:22" x14ac:dyDescent="0.25">
       <c r="P61" s="116"/>
     </row>
-    <row r="62" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B62" s="129" t="s">
         <v>148</v>
       </c>
@@ -18745,7 +19011,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="63" spans="2:22" ht="58" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:22" ht="75" x14ac:dyDescent="0.25">
       <c r="B63" s="21" t="s">
         <v>48</v>
       </c>
@@ -18789,7 +19055,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="64" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B64" s="21">
         <v>1</v>
       </c>
@@ -18839,7 +19105,7 @@
         <v>4.8626492370267685E-2</v>
       </c>
     </row>
-    <row r="65" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B65" s="21">
         <v>2</v>
       </c>
@@ -18889,7 +19155,7 @@
         <v>4.0808325124378882E-2</v>
       </c>
     </row>
-    <row r="66" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B66" s="21">
         <v>3</v>
       </c>
@@ -18939,7 +19205,7 @@
         <v>3.6317916629681209E-2</v>
       </c>
     </row>
-    <row r="67" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B67" s="21">
         <v>4</v>
       </c>
@@ -18989,7 +19255,7 @@
         <v>3.2970622516849388E-2</v>
       </c>
     </row>
-    <row r="68" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B68" s="21">
         <v>5</v>
       </c>
@@ -19039,7 +19305,7 @@
         <v>3.0407676295365581E-2</v>
       </c>
     </row>
-    <row r="69" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B69" s="21">
         <v>6</v>
       </c>
@@ -19089,7 +19355,7 @@
         <v>2.7949066295852726E-2</v>
       </c>
     </row>
-    <row r="70" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B70" s="21">
         <v>7</v>
       </c>
@@ -19139,7 +19405,7 @@
         <v>2.5821637832360165E-2</v>
       </c>
     </row>
-    <row r="71" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B71" s="21">
         <v>8</v>
       </c>
@@ -19189,7 +19455,7 @@
         <v>2.298055159816071E-2</v>
       </c>
     </row>
-    <row r="72" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B72" s="21">
         <v>9</v>
       </c>
@@ -19239,7 +19505,7 @@
         <v>2.0441022189923958E-2</v>
       </c>
     </row>
-    <row r="73" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B73" s="21">
         <v>10</v>
       </c>
@@ -19289,7 +19555,7 @@
         <v>1.4752059212155852E-2</v>
       </c>
     </row>
-    <row r="76" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B76" s="129" t="s">
         <v>149</v>
       </c>
@@ -19303,7 +19569,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="77" spans="2:22" ht="58" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:22" ht="75" x14ac:dyDescent="0.25">
       <c r="B77" s="21" t="s">
         <v>48</v>
       </c>
@@ -19347,7 +19613,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="78" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B78" s="21">
         <v>1</v>
       </c>
@@ -19397,7 +19663,7 @@
         <v>4.6220878177670455E-2</v>
       </c>
     </row>
-    <row r="79" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B79" s="21">
         <v>2</v>
       </c>
@@ -19447,7 +19713,7 @@
         <v>3.8785485016665497E-2</v>
       </c>
     </row>
-    <row r="80" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B80" s="21">
         <v>3</v>
       </c>
@@ -19497,7 +19763,7 @@
         <v>3.522958664864255E-2</v>
       </c>
     </row>
-    <row r="81" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B81" s="21">
         <v>4</v>
       </c>
@@ -19547,7 +19813,7 @@
         <v>3.2758089561005496E-2</v>
       </c>
     </row>
-    <row r="82" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B82" s="21">
         <v>5</v>
       </c>
@@ -19597,7 +19863,7 @@
         <v>3.0813517572023157E-2</v>
       </c>
     </row>
-    <row r="83" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B83" s="21">
         <v>6</v>
       </c>
@@ -19647,7 +19913,7 @@
         <v>2.9273945299745318E-2</v>
       </c>
     </row>
-    <row r="84" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B84" s="21">
         <v>7</v>
       </c>
@@ -19697,7 +19963,7 @@
         <v>2.7525475176612926E-2</v>
       </c>
     </row>
-    <row r="85" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B85" s="21">
         <v>8</v>
       </c>
@@ -19747,7 +20013,7 @@
         <v>2.413582523534941E-2</v>
       </c>
     </row>
-    <row r="86" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B86" s="21">
         <v>9</v>
       </c>
@@ -19797,7 +20063,7 @@
         <v>2.3299360859623707E-2</v>
       </c>
     </row>
-    <row r="87" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B87" s="21">
         <v>10</v>
       </c>
@@ -19847,7 +20113,7 @@
         <v>1.5299585052049499E-2</v>
       </c>
     </row>
-    <row r="90" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B90" s="129" t="s">
         <v>152</v>
       </c>
@@ -19861,7 +20127,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="91" spans="2:22" ht="58" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:22" ht="75" x14ac:dyDescent="0.25">
       <c r="B91" s="21" t="s">
         <v>48</v>
       </c>
@@ -19905,7 +20171,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="92" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B92" s="21">
         <v>1</v>
       </c>
@@ -19955,7 +20221,7 @@
         <v>4.8157489034379136E-2</v>
       </c>
     </row>
-    <row r="93" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B93" s="21">
         <v>2</v>
       </c>
@@ -20005,7 +20271,7 @@
         <v>4.0588053137738105E-2</v>
       </c>
     </row>
-    <row r="94" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B94" s="21">
         <v>3</v>
       </c>
@@ -20055,7 +20321,7 @@
         <v>3.623693482688764E-2</v>
       </c>
     </row>
-    <row r="95" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B95" s="21">
         <v>4</v>
       </c>
@@ -20105,7 +20371,7 @@
         <v>3.2959805886672362E-2</v>
       </c>
     </row>
-    <row r="96" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B96" s="21">
         <v>5</v>
       </c>
@@ -20155,7 +20421,7 @@
         <v>3.0421824003404423E-2</v>
       </c>
     </row>
-    <row r="97" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B97" s="21">
         <v>6</v>
       </c>
@@ -20205,7 +20471,7 @@
         <v>2.7981360308230348E-2</v>
       </c>
     </row>
-    <row r="98" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B98" s="21">
         <v>7</v>
       </c>
@@ -20255,7 +20521,7 @@
         <v>2.5856945692073047E-2</v>
       </c>
     </row>
-    <row r="99" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B99" s="21">
         <v>8</v>
       </c>
@@ -20305,7 +20571,7 @@
         <v>2.2998179618774733E-2</v>
       </c>
     </row>
-    <row r="100" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B100" s="21">
         <v>9</v>
       </c>
@@ -20355,7 +20621,7 @@
         <v>2.0465725263592568E-2</v>
       </c>
     </row>
-    <row r="101" spans="2:22" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B101" s="21">
         <v>10</v>
       </c>

</xml_diff>